<commit_message>
Publish Tacen_2016_WC, Tacen_2023_WC, Tacen_2025_WC, Tacen_2026_WC
</commit_message>
<xml_diff>
--- a/events/Tacen_2016_WC/Tacen_2016_WC_start.xlsx
+++ b/events/Tacen_2016_WC/Tacen_2016_WC_start.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W553"/>
+  <dimension ref="A1:AC553"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,17 +519,47 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
+          <t>Name4</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Name5</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Name6</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>ICF_ID1</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>ICF_ID2</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>ICF_ID3</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>ICF_ID4</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>ICF_ID5</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>ICF_ID6</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1312,7 @@
           <t>SASAKI Suguru</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>69002</t>
         </is>
@@ -1340,7 +1370,7 @@
           <t>LOWTHER Steven</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="X17" t="inlineStr">
         <is>
           <t>44811</t>
         </is>
@@ -1398,7 +1428,7 @@
           <t>CRAWFORD Brodie</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="X18" t="inlineStr">
         <is>
           <t>38436</t>
         </is>
@@ -1456,7 +1486,7 @@
           <t>McEWAN Devin</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="X19" t="inlineStr">
         <is>
           <t>35068</t>
         </is>
@@ -1514,7 +1544,7 @@
           <t>MARZO Daniel</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>35757</t>
         </is>
@@ -1572,7 +1602,7 @@
           <t>LAVIOLETTE Yannick</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>43343</t>
         </is>
@@ -1630,7 +1660,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="X22" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -1688,7 +1718,7 @@
           <t>POMEROY Spencer</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>57783</t>
         </is>
@@ -1746,7 +1776,7 @@
           <t>WATKINS Daniel</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>38430</t>
         </is>
@@ -1804,7 +1834,7 @@
           <t>TRAVE Miquel</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="X25" t="inlineStr">
         <is>
           <t>68998</t>
         </is>
@@ -1862,7 +1892,7 @@
           <t>PLEWA Przemyslaw</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="X26" t="inlineStr">
         <is>
           <t>35950</t>
         </is>
@@ -1920,7 +1950,7 @@
           <t>HENDRICK Robert</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="X27" t="inlineStr">
         <is>
           <t>43002</t>
         </is>
@@ -1978,7 +2008,7 @@
           <t>TEBE Jordi</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="X28" t="inlineStr">
         <is>
           <t>51853</t>
         </is>
@@ -2036,7 +2066,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="X29" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -2094,7 +2124,7 @@
           <t>SOETER Dennis</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="X30" t="inlineStr">
         <is>
           <t>39166</t>
         </is>
@@ -2152,7 +2182,7 @@
           <t>CORREA Charles</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
+      <c r="X31" t="inlineStr">
         <is>
           <t>38018</t>
         </is>
@@ -2210,7 +2240,7 @@
           <t>SHU Jianming</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="X32" t="inlineStr">
         <is>
           <t>47327</t>
         </is>
@@ -2268,7 +2298,7 @@
           <t>FOULON Kilian</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
+      <c r="X33" t="inlineStr">
         <is>
           <t>35602</t>
         </is>
@@ -2326,7 +2356,7 @@
           <t>BADURA Jergus</t>
         </is>
       </c>
-      <c r="U34" t="inlineStr">
+      <c r="X34" t="inlineStr">
         <is>
           <t>68767</t>
         </is>
@@ -2384,7 +2414,7 @@
           <t>CHOOAMPAI Rattanajet</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
+      <c r="X35" t="inlineStr">
         <is>
           <t>51801</t>
         </is>
@@ -2442,7 +2472,7 @@
           <t>CHAIDET Yutthakan</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
+      <c r="X36" t="inlineStr">
         <is>
           <t>51798</t>
         </is>
@@ -2500,7 +2530,7 @@
           <t>SASAKI Shota</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr">
+      <c r="X37" t="inlineStr">
         <is>
           <t>41610</t>
         </is>
@@ -2558,7 +2588,7 @@
           <t>SMEDLEY Liam</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
+      <c r="X38" t="inlineStr">
         <is>
           <t>36517</t>
         </is>
@@ -2669,7 +2699,7 @@
           <t>GIBB Benjamin</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
+      <c r="X40" t="inlineStr">
         <is>
           <t>36711</t>
         </is>
@@ -2727,7 +2757,7 @@
           <t>BORGES Felipe</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="X41" t="inlineStr">
         <is>
           <t>38012</t>
         </is>
@@ -2785,7 +2815,7 @@
           <t>CECCON Paolo</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="X42" t="inlineStr">
         <is>
           <t>39903</t>
         </is>
@@ -2843,7 +2873,7 @@
           <t>IVALDI Raffaello</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="X43" t="inlineStr">
         <is>
           <t>35227</t>
         </is>
@@ -2901,7 +2931,7 @@
           <t>JEGOU Liam</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr">
+      <c r="X44" t="inlineStr">
         <is>
           <t>35820</t>
         </is>
@@ -2959,7 +2989,7 @@
           <t>COF Blaz</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr">
+      <c r="X45" t="inlineStr">
         <is>
           <t>36897</t>
         </is>
@@ -3017,7 +3047,7 @@
           <t>HEDWIG Grzegorz</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="X46" t="inlineStr">
         <is>
           <t>35465</t>
         </is>
@@ -3075,7 +3105,7 @@
           <t>COLAZINGARI Roberto</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="X47" t="inlineStr">
         <is>
           <t>35223</t>
         </is>
@@ -3133,7 +3163,7 @@
           <t>BETTGE Nico</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="X48" t="inlineStr">
         <is>
           <t>35133</t>
         </is>
@@ -3191,7 +3221,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
+      <c r="X49" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -3249,7 +3279,7 @@
           <t>MARINIC Matija</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr">
+      <c r="X50" t="inlineStr">
         <is>
           <t>35595</t>
         </is>
@@ -3307,7 +3337,7 @@
           <t>BREUER Florian</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr">
+      <c r="X51" t="inlineStr">
         <is>
           <t>39171</t>
         </is>
@@ -3365,7 +3395,7 @@
           <t>THOMAS Martin</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
+      <c r="X52" t="inlineStr">
         <is>
           <t>35412</t>
         </is>
@@ -3423,7 +3453,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr">
+      <c r="X53" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -3481,7 +3511,7 @@
           <t>BURGESS Adam</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr">
+      <c r="X54" t="inlineStr">
         <is>
           <t>35647</t>
         </is>
@@ -3539,7 +3569,7 @@
           <t>WESTLEY Ryan</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr">
+      <c r="X55" t="inlineStr">
         <is>
           <t>35651</t>
         </is>
@@ -3597,7 +3627,7 @@
           <t>LENARCIC Jure</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
+      <c r="X56" t="inlineStr">
         <is>
           <t>36259</t>
         </is>
@@ -3655,7 +3685,7 @@
           <t>TILLARD Pierre-Antoine</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr">
+      <c r="X57" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
@@ -3713,7 +3743,7 @@
           <t>GEBAS Vitezslav</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr">
+      <c r="X58" t="inlineStr">
         <is>
           <t>35038</t>
         </is>
@@ -3771,7 +3801,7 @@
           <t>PESCHIER Nicolas</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
+      <c r="X59" t="inlineStr">
         <is>
           <t>35401</t>
         </is>
@@ -3829,7 +3859,7 @@
           <t>EICHFELD Casey</t>
         </is>
       </c>
-      <c r="U60" t="inlineStr">
+      <c r="X60" t="inlineStr">
         <is>
           <t>35067</t>
         </is>
@@ -3887,7 +3917,7 @@
           <t>KOECHLIN Thomas</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr">
+      <c r="X61" t="inlineStr">
         <is>
           <t>35419</t>
         </is>
@@ -3945,7 +3975,7 @@
           <t>BERCIC Anze</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
+      <c r="X62" t="inlineStr">
         <is>
           <t>36253</t>
         </is>
@@ -4003,7 +4033,7 @@
           <t>ANTON Franz</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
+      <c r="X63" t="inlineStr">
         <is>
           <t>35137</t>
         </is>
@@ -4061,7 +4091,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr">
+      <c r="X64" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -4119,7 +4149,7 @@
           <t>BENUS Matej</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr">
+      <c r="X65" t="inlineStr">
         <is>
           <t>35353</t>
         </is>
@@ -4177,7 +4207,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr">
+      <c r="X66" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -4235,7 +4265,7 @@
           <t>ZHANG Jinjie</t>
         </is>
       </c>
-      <c r="U67" t="inlineStr">
+      <c r="X67" t="inlineStr">
         <is>
           <t>72213</t>
         </is>
@@ -4293,7 +4323,7 @@
           <t>WALL Demelza</t>
         </is>
       </c>
-      <c r="U68" t="inlineStr">
+      <c r="X68" t="inlineStr">
         <is>
           <t>60107</t>
         </is>
@@ -4351,7 +4381,7 @@
           <t>O'FERRALL Caoimhe</t>
         </is>
       </c>
-      <c r="U69" t="inlineStr">
+      <c r="X69" t="inlineStr">
         <is>
           <t>61007</t>
         </is>
@@ -4409,7 +4439,7 @@
           <t>NOVAK Lea</t>
         </is>
       </c>
-      <c r="U70" t="inlineStr">
+      <c r="X70" t="inlineStr">
         <is>
           <t>60323</t>
         </is>
@@ -4467,7 +4497,7 @@
           <t>YAGI Airi</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr">
+      <c r="X71" t="inlineStr">
         <is>
           <t>37756</t>
         </is>
@@ -4525,7 +4555,7 @@
           <t>BETTERIDGE Lois</t>
         </is>
       </c>
-      <c r="U72" t="inlineStr">
+      <c r="X72" t="inlineStr">
         <is>
           <t>60078</t>
         </is>
@@ -4583,7 +4613,7 @@
           <t>DUANGLAWA Atcharaporn</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr">
+      <c r="X73" t="inlineStr">
         <is>
           <t>61799</t>
         </is>
@@ -4641,7 +4671,7 @@
           <t>SATO Ayano</t>
         </is>
       </c>
-      <c r="U74" t="inlineStr">
+      <c r="X74" t="inlineStr">
         <is>
           <t>60374</t>
         </is>
@@ -4752,7 +4782,7 @@
           <t>NAVEAU Laurine</t>
         </is>
       </c>
-      <c r="U76" t="inlineStr">
+      <c r="X76" t="inlineStr">
         <is>
           <t>53246</t>
         </is>
@@ -4810,7 +4840,7 @@
           <t>KOZOROG Alja</t>
         </is>
       </c>
-      <c r="U77" t="inlineStr">
+      <c r="X77" t="inlineStr">
         <is>
           <t>39986</t>
         </is>
@@ -4868,7 +4898,7 @@
           <t>GLEJTEKOVA Simona</t>
         </is>
       </c>
-      <c r="U78" t="inlineStr">
+      <c r="X78" t="inlineStr">
         <is>
           <t>55166</t>
         </is>
@@ -4979,7 +5009,7 @@
           <t>MACEKOVA Simona</t>
         </is>
       </c>
-      <c r="U80" t="inlineStr">
+      <c r="X80" t="inlineStr">
         <is>
           <t>45153</t>
         </is>
@@ -5037,7 +5067,7 @@
           <t>BIZJAK Nina</t>
         </is>
       </c>
-      <c r="U81" t="inlineStr">
+      <c r="X81" t="inlineStr">
         <is>
           <t>39984</t>
         </is>
@@ -5095,7 +5125,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U82" t="inlineStr">
+      <c r="X82" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -5153,7 +5183,7 @@
           <t>STANOVSKA Sona</t>
         </is>
       </c>
-      <c r="U83" t="inlineStr">
+      <c r="X83" t="inlineStr">
         <is>
           <t>51647</t>
         </is>
@@ -5211,7 +5241,7 @@
           <t>JANCZY Justyna</t>
         </is>
       </c>
-      <c r="U84" t="inlineStr">
+      <c r="X84" t="inlineStr">
         <is>
           <t>43975</t>
         </is>
@@ -5269,7 +5299,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U85" t="inlineStr">
+      <c r="X85" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -5327,7 +5357,7 @@
           <t>MATULKOVA Jana</t>
         </is>
       </c>
-      <c r="U86" t="inlineStr">
+      <c r="X86" t="inlineStr">
         <is>
           <t>37274</t>
         </is>
@@ -5385,7 +5415,7 @@
           <t>TIXIER Cecile</t>
         </is>
       </c>
-      <c r="U87" t="inlineStr">
+      <c r="X87" t="inlineStr">
         <is>
           <t>35687</t>
         </is>
@@ -5443,7 +5473,7 @@
           <t>PRIOUX Lucie</t>
         </is>
       </c>
-      <c r="U88" t="inlineStr">
+      <c r="X88" t="inlineStr">
         <is>
           <t>42984</t>
         </is>
@@ -5501,7 +5531,7 @@
           <t>WERATSCHNIG Nadine</t>
         </is>
       </c>
-      <c r="U89" t="inlineStr">
+      <c r="X89" t="inlineStr">
         <is>
           <t>41613</t>
         </is>
@@ -5612,7 +5642,7 @@
           <t>VAN DER KNIJFF Annebel</t>
         </is>
       </c>
-      <c r="U91" t="inlineStr">
+      <c r="X91" t="inlineStr">
         <is>
           <t>39945</t>
         </is>
@@ -5670,7 +5700,7 @@
           <t>GIBSON Eilidh</t>
         </is>
       </c>
-      <c r="U92" t="inlineStr">
+      <c r="X92" t="inlineStr">
         <is>
           <t>36708</t>
         </is>
@@ -5728,7 +5758,7 @@
           <t>JACQUET Claire</t>
         </is>
       </c>
-      <c r="U93" t="inlineStr">
+      <c r="X93" t="inlineStr">
         <is>
           <t>35684</t>
         </is>
@@ -5839,7 +5869,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U95" t="inlineStr">
+      <c r="X95" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -5897,7 +5927,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U96" t="inlineStr">
+      <c r="X96" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -5955,7 +5985,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U97" t="inlineStr">
+      <c r="X97" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -6013,7 +6043,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U98" t="inlineStr">
+      <c r="X98" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -6071,7 +6101,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U99" t="inlineStr">
+      <c r="X99" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -6129,7 +6159,7 @@
           <t>LAUNAY Damien</t>
         </is>
       </c>
-      <c r="U100" t="inlineStr">
+      <c r="X100" t="inlineStr">
         <is>
           <t>60047</t>
         </is>
@@ -6187,7 +6217,7 @@
           <t>SIMPSON Keenan</t>
         </is>
       </c>
-      <c r="U101" t="inlineStr">
+      <c r="X101" t="inlineStr">
         <is>
           <t>71797</t>
         </is>
@@ -6245,7 +6275,7 @@
           <t>MUSGRAVE Andrew</t>
         </is>
       </c>
-      <c r="U102" t="inlineStr">
+      <c r="X102" t="inlineStr">
         <is>
           <t>60102</t>
         </is>
@@ -6303,7 +6333,7 @@
           <t>HENDRICK Noel</t>
         </is>
       </c>
-      <c r="U103" t="inlineStr">
+      <c r="X103" t="inlineStr">
         <is>
           <t>43003</t>
         </is>
@@ -6361,7 +6391,7 @@
           <t>STOILJKOVIC Dusan</t>
         </is>
       </c>
-      <c r="U104" t="inlineStr">
+      <c r="X104" t="inlineStr">
         <is>
           <t>35791</t>
         </is>
@@ -6419,7 +6449,7 @@
           <t>BOWERS Christopher</t>
         </is>
       </c>
-      <c r="U105" t="inlineStr">
+      <c r="X105" t="inlineStr">
         <is>
           <t>52010</t>
         </is>
@@ -6477,7 +6507,7 @@
           <t>KORPES Ren</t>
         </is>
       </c>
-      <c r="U106" t="inlineStr">
+      <c r="X106" t="inlineStr">
         <is>
           <t>39941</t>
         </is>
@@ -6535,7 +6565,7 @@
           <t>SASAKI Tsubasa Terry</t>
         </is>
       </c>
-      <c r="U107" t="inlineStr">
+      <c r="X107" t="inlineStr">
         <is>
           <t>47085</t>
         </is>
@@ -6593,7 +6623,7 @@
           <t>MAIKRANZ Alexandr</t>
         </is>
       </c>
-      <c r="U108" t="inlineStr">
+      <c r="X108" t="inlineStr">
         <is>
           <t>60018</t>
         </is>
@@ -6651,7 +6681,7 @@
           <t>TRAVOSTINO Benjamin</t>
         </is>
       </c>
-      <c r="U109" t="inlineStr">
+      <c r="X109" t="inlineStr">
         <is>
           <t>68795</t>
         </is>
@@ -6709,7 +6739,7 @@
           <t>SANDERA Wiktor</t>
         </is>
       </c>
-      <c r="U110" t="inlineStr">
+      <c r="X110" t="inlineStr">
         <is>
           <t>53642</t>
         </is>
@@ -6767,7 +6797,7 @@
           <t>LEE EDWARDS Ciaran</t>
         </is>
       </c>
-      <c r="U111" t="inlineStr">
+      <c r="X111" t="inlineStr">
         <is>
           <t>35614</t>
         </is>
@@ -6825,7 +6855,7 @@
           <t>LLORENTE David</t>
         </is>
       </c>
-      <c r="U112" t="inlineStr">
+      <c r="X112" t="inlineStr">
         <is>
           <t>51850</t>
         </is>
@@ -6883,7 +6913,7 @@
           <t>CURTIS Samuel</t>
         </is>
       </c>
-      <c r="U113" t="inlineStr">
+      <c r="X113" t="inlineStr">
         <is>
           <t>36683</t>
         </is>
@@ -6941,7 +6971,7 @@
           <t>KANAYA Tohru</t>
         </is>
       </c>
-      <c r="U114" t="inlineStr">
+      <c r="X114" t="inlineStr">
         <is>
           <t>36484</t>
         </is>
@@ -6999,7 +7029,7 @@
           <t>POPE Benjamin</t>
         </is>
       </c>
-      <c r="U115" t="inlineStr">
+      <c r="X115" t="inlineStr">
         <is>
           <t>51753</t>
         </is>
@@ -7057,7 +7087,7 @@
           <t>MUNSCH Manuel</t>
         </is>
       </c>
-      <c r="U116" t="inlineStr">
+      <c r="X116" t="inlineStr">
         <is>
           <t>35631</t>
         </is>
@@ -7115,7 +7145,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U117" t="inlineStr">
+      <c r="X117" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -7173,7 +7203,7 @@
           <t>BEDA Marcello</t>
         </is>
       </c>
-      <c r="U118" t="inlineStr">
+      <c r="X118" t="inlineStr">
         <is>
           <t>39899</t>
         </is>
@@ -7231,7 +7261,7 @@
           <t>TAN Ya</t>
         </is>
       </c>
-      <c r="U119" t="inlineStr">
+      <c r="X119" t="inlineStr">
         <is>
           <t>52024</t>
         </is>
@@ -7289,7 +7319,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U120" t="inlineStr">
+      <c r="X120" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -7347,7 +7377,7 @@
           <t>ANDERSON Timothy</t>
         </is>
       </c>
-      <c r="U121" t="inlineStr">
+      <c r="X121" t="inlineStr">
         <is>
           <t>38432</t>
         </is>
@@ -7405,7 +7435,7 @@
           <t>WEGER Matthias</t>
         </is>
       </c>
-      <c r="U122" t="inlineStr">
+      <c r="X122" t="inlineStr">
         <is>
           <t>68837</t>
         </is>
@@ -7463,7 +7493,7 @@
           <t>CADENA Jordi</t>
         </is>
       </c>
-      <c r="U123" t="inlineStr">
+      <c r="X123" t="inlineStr">
         <is>
           <t>41644</t>
         </is>
@@ -7521,7 +7551,7 @@
           <t>BUTCHER Finn</t>
         </is>
       </c>
-      <c r="U124" t="inlineStr">
+      <c r="X124" t="inlineStr">
         <is>
           <t>36663</t>
         </is>
@@ -7579,7 +7609,7 @@
           <t>ADACHI Kazuya</t>
         </is>
       </c>
-      <c r="U125" t="inlineStr">
+      <c r="X125" t="inlineStr">
         <is>
           <t>36646</t>
         </is>
@@ -7637,7 +7667,7 @@
           <t>WATKINS Daniel</t>
         </is>
       </c>
-      <c r="U126" t="inlineStr">
+      <c r="X126" t="inlineStr">
         <is>
           <t>38430</t>
         </is>
@@ -7695,7 +7725,7 @@
           <t>HOLMER Erik</t>
         </is>
       </c>
-      <c r="U127" t="inlineStr">
+      <c r="X127" t="inlineStr">
         <is>
           <t>35104</t>
         </is>
@@ -7753,7 +7783,7 @@
           <t>TAYLER Michael</t>
         </is>
       </c>
-      <c r="U128" t="inlineStr">
+      <c r="X128" t="inlineStr">
         <is>
           <t>36262</t>
         </is>
@@ -7811,7 +7841,7 @@
           <t>DOUGOUD Martin</t>
         </is>
       </c>
-      <c r="U129" t="inlineStr">
+      <c r="X129" t="inlineStr">
         <is>
           <t>35426</t>
         </is>
@@ -7922,7 +7952,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U131" t="inlineStr">
+      <c r="X131" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -7980,7 +8010,7 @@
           <t>IVALDI Zeno</t>
         </is>
       </c>
-      <c r="U132" t="inlineStr">
+      <c r="X132" t="inlineStr">
         <is>
           <t>35480</t>
         </is>
@@ -8038,7 +8068,7 @@
           <t>POTOCNY Marcel</t>
         </is>
       </c>
-      <c r="U133" t="inlineStr">
+      <c r="X133" t="inlineStr">
         <is>
           <t>35235</t>
         </is>
@@ -8096,7 +8126,7 @@
           <t>HUJSA Matus</t>
         </is>
       </c>
-      <c r="U134" t="inlineStr">
+      <c r="X134" t="inlineStr">
         <is>
           <t>35503</t>
         </is>
@@ -8154,7 +8184,7 @@
           <t>MAXEINER Tim</t>
         </is>
       </c>
-      <c r="U135" t="inlineStr">
+      <c r="X135" t="inlineStr">
         <is>
           <t>35117</t>
         </is>
@@ -8212,7 +8242,7 @@
           <t>OSCHMAUTZ Felix</t>
         </is>
       </c>
-      <c r="U136" t="inlineStr">
+      <c r="X136" t="inlineStr">
         <is>
           <t>51856</t>
         </is>
@@ -8270,7 +8300,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U137" t="inlineStr">
+      <c r="X137" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -8381,7 +8411,7 @@
           <t>SRABOTNIK Martin</t>
         </is>
       </c>
-      <c r="U139" t="inlineStr">
+      <c r="X139" t="inlineStr">
         <is>
           <t>39080</t>
         </is>
@@ -8439,7 +8469,7 @@
           <t>MALEK Andrej</t>
         </is>
       </c>
-      <c r="U140" t="inlineStr">
+      <c r="X140" t="inlineStr">
         <is>
           <t>39246</t>
         </is>
@@ -8497,7 +8527,7 @@
           <t>BOECKELMANN Paul</t>
         </is>
       </c>
-      <c r="U141" t="inlineStr">
+      <c r="X141" t="inlineStr">
         <is>
           <t>35118</t>
         </is>
@@ -8555,7 +8585,7 @@
           <t>FORBES-CRYANS Bradley</t>
         </is>
       </c>
-      <c r="U142" t="inlineStr">
+      <c r="X142" t="inlineStr">
         <is>
           <t>36513</t>
         </is>
@@ -8613,7 +8643,7 @@
           <t>MEGLIC Jure</t>
         </is>
       </c>
-      <c r="U143" t="inlineStr">
+      <c r="X143" t="inlineStr">
         <is>
           <t>35590</t>
         </is>
@@ -8671,7 +8701,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U144" t="inlineStr">
+      <c r="X144" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -8729,7 +8759,7 @@
           <t>ALBREHT Martin</t>
         </is>
       </c>
-      <c r="U145" t="inlineStr">
+      <c r="X145" t="inlineStr">
         <is>
           <t>36898</t>
         </is>
@@ -8787,7 +8817,7 @@
           <t>OKREGLAK Maciej</t>
         </is>
       </c>
-      <c r="U146" t="inlineStr">
+      <c r="X146" t="inlineStr">
         <is>
           <t>35088</t>
         </is>
@@ -8845,7 +8875,7 @@
           <t>DAILLE Etienne</t>
         </is>
       </c>
-      <c r="U147" t="inlineStr">
+      <c r="X147" t="inlineStr">
         <is>
           <t>35308</t>
         </is>
@@ -8903,7 +8933,7 @@
           <t>BOURLIAUD Pierre</t>
         </is>
       </c>
-      <c r="U148" t="inlineStr">
+      <c r="X148" t="inlineStr">
         <is>
           <t>35230</t>
         </is>
@@ -8961,7 +8991,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U149" t="inlineStr">
+      <c r="X149" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -9019,7 +9049,7 @@
           <t>HILGERT Lubos</t>
         </is>
       </c>
-      <c r="U150" t="inlineStr">
+      <c r="X150" t="inlineStr">
         <is>
           <t>35032</t>
         </is>
@@ -9077,7 +9107,7 @@
           <t>DE GENNARO Giovanni</t>
         </is>
       </c>
-      <c r="U151" t="inlineStr">
+      <c r="X151" t="inlineStr">
         <is>
           <t>35244</t>
         </is>
@@ -9135,7 +9165,7 @@
           <t>TUNKA Ondrej</t>
         </is>
       </c>
-      <c r="U152" t="inlineStr">
+      <c r="X152" t="inlineStr">
         <is>
           <t>35947</t>
         </is>
@@ -9193,7 +9223,7 @@
           <t>GRIMM Alexander</t>
         </is>
       </c>
-      <c r="U153" t="inlineStr">
+      <c r="X153" t="inlineStr">
         <is>
           <t>35112</t>
         </is>
@@ -9251,7 +9281,7 @@
           <t>POPIELA Dariusz</t>
         </is>
       </c>
-      <c r="U154" t="inlineStr">
+      <c r="X154" t="inlineStr">
         <is>
           <t>35096</t>
         </is>
@@ -9309,7 +9339,7 @@
           <t>PRINDIS Vit</t>
         </is>
       </c>
-      <c r="U155" t="inlineStr">
+      <c r="X155" t="inlineStr">
         <is>
           <t>35065</t>
         </is>
@@ -9367,7 +9397,7 @@
           <t>GRIGAR Jakub</t>
         </is>
       </c>
-      <c r="U156" t="inlineStr">
+      <c r="X156" t="inlineStr">
         <is>
           <t>37284</t>
         </is>
@@ -9425,7 +9455,7 @@
           <t>POLACZYK Mateusz</t>
         </is>
       </c>
-      <c r="U157" t="inlineStr">
+      <c r="X157" t="inlineStr">
         <is>
           <t>35072</t>
         </is>
@@ -9483,7 +9513,7 @@
           <t>SCHUBERT Sebastian</t>
         </is>
       </c>
-      <c r="U158" t="inlineStr">
+      <c r="X158" t="inlineStr">
         <is>
           <t>35114</t>
         </is>
@@ -9541,7 +9571,7 @@
           <t>BERSINGER Thomas</t>
         </is>
       </c>
-      <c r="U159" t="inlineStr">
+      <c r="X159" t="inlineStr">
         <is>
           <t>35228</t>
         </is>
@@ -9599,7 +9629,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U160" t="inlineStr">
+      <c r="X160" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -9657,7 +9687,7 @@
           <t>HERNANZ Samuel</t>
         </is>
       </c>
-      <c r="U161" t="inlineStr">
+      <c r="X161" t="inlineStr">
         <is>
           <t>35786</t>
         </is>
@@ -9715,7 +9745,7 @@
           <t>BIAZIZZO Mathieu</t>
         </is>
       </c>
-      <c r="U162" t="inlineStr">
+      <c r="X162" t="inlineStr">
         <is>
           <t>35484</t>
         </is>
@@ -9773,7 +9803,7 @@
           <t>NEVEU Boris</t>
         </is>
       </c>
-      <c r="U163" t="inlineStr">
+      <c r="X163" t="inlineStr">
         <is>
           <t>35396</t>
         </is>
@@ -9831,7 +9861,7 @@
           <t>SASAKI Suguru</t>
         </is>
       </c>
-      <c r="U164" t="inlineStr">
+      <c r="X164" t="inlineStr">
         <is>
           <t>69002</t>
         </is>
@@ -9889,7 +9919,7 @@
           <t>LOWTHER Steven</t>
         </is>
       </c>
-      <c r="U165" t="inlineStr">
+      <c r="X165" t="inlineStr">
         <is>
           <t>44811</t>
         </is>
@@ -9947,7 +9977,7 @@
           <t>CRAWFORD Brodie</t>
         </is>
       </c>
-      <c r="U166" t="inlineStr">
+      <c r="X166" t="inlineStr">
         <is>
           <t>38436</t>
         </is>
@@ -10005,7 +10035,7 @@
           <t>McEWAN Devin</t>
         </is>
       </c>
-      <c r="U167" t="inlineStr">
+      <c r="X167" t="inlineStr">
         <is>
           <t>35068</t>
         </is>
@@ -10063,7 +10093,7 @@
           <t>MARZO Daniel</t>
         </is>
       </c>
-      <c r="U168" t="inlineStr">
+      <c r="X168" t="inlineStr">
         <is>
           <t>35757</t>
         </is>
@@ -10121,7 +10151,7 @@
           <t>LAVIOLETTE Yannick</t>
         </is>
       </c>
-      <c r="U169" t="inlineStr">
+      <c r="X169" t="inlineStr">
         <is>
           <t>43343</t>
         </is>
@@ -10179,7 +10209,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U170" t="inlineStr">
+      <c r="X170" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -10237,7 +10267,7 @@
           <t>POMEROY Spencer</t>
         </is>
       </c>
-      <c r="U171" t="inlineStr">
+      <c r="X171" t="inlineStr">
         <is>
           <t>57783</t>
         </is>
@@ -10295,7 +10325,7 @@
           <t>WATKINS Daniel</t>
         </is>
       </c>
-      <c r="U172" t="inlineStr">
+      <c r="X172" t="inlineStr">
         <is>
           <t>38430</t>
         </is>
@@ -10353,7 +10383,7 @@
           <t>TRAVE Miquel</t>
         </is>
       </c>
-      <c r="U173" t="inlineStr">
+      <c r="X173" t="inlineStr">
         <is>
           <t>68998</t>
         </is>
@@ -10411,7 +10441,7 @@
           <t>PLEWA Przemyslaw</t>
         </is>
       </c>
-      <c r="U174" t="inlineStr">
+      <c r="X174" t="inlineStr">
         <is>
           <t>35950</t>
         </is>
@@ -10469,7 +10499,7 @@
           <t>HENDRICK Robert</t>
         </is>
       </c>
-      <c r="U175" t="inlineStr">
+      <c r="X175" t="inlineStr">
         <is>
           <t>43002</t>
         </is>
@@ -10527,7 +10557,7 @@
           <t>TEBE Jordi</t>
         </is>
       </c>
-      <c r="U176" t="inlineStr">
+      <c r="X176" t="inlineStr">
         <is>
           <t>51853</t>
         </is>
@@ -10585,7 +10615,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U177" t="inlineStr">
+      <c r="X177" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -10643,7 +10673,7 @@
           <t>SOETER Dennis</t>
         </is>
       </c>
-      <c r="U178" t="inlineStr">
+      <c r="X178" t="inlineStr">
         <is>
           <t>39166</t>
         </is>
@@ -10701,7 +10731,7 @@
           <t>CORREA Charles</t>
         </is>
       </c>
-      <c r="U179" t="inlineStr">
+      <c r="X179" t="inlineStr">
         <is>
           <t>38018</t>
         </is>
@@ -10759,7 +10789,7 @@
           <t>SHU Jianming</t>
         </is>
       </c>
-      <c r="U180" t="inlineStr">
+      <c r="X180" t="inlineStr">
         <is>
           <t>47327</t>
         </is>
@@ -10817,7 +10847,7 @@
           <t>FOULON Kilian</t>
         </is>
       </c>
-      <c r="U181" t="inlineStr">
+      <c r="X181" t="inlineStr">
         <is>
           <t>35602</t>
         </is>
@@ -10875,7 +10905,7 @@
           <t>CHOOAMPAI Rattanajet</t>
         </is>
       </c>
-      <c r="U182" t="inlineStr">
+      <c r="X182" t="inlineStr">
         <is>
           <t>51801</t>
         </is>
@@ -10933,7 +10963,7 @@
           <t>CHAIDET Yutthakan</t>
         </is>
       </c>
-      <c r="U183" t="inlineStr">
+      <c r="X183" t="inlineStr">
         <is>
           <t>51798</t>
         </is>
@@ -10991,7 +11021,7 @@
           <t>SASAKI Shota</t>
         </is>
       </c>
-      <c r="U184" t="inlineStr">
+      <c r="X184" t="inlineStr">
         <is>
           <t>41610</t>
         </is>
@@ -11049,7 +11079,7 @@
           <t>SMEDLEY Liam</t>
         </is>
       </c>
-      <c r="U185" t="inlineStr">
+      <c r="X185" t="inlineStr">
         <is>
           <t>36517</t>
         </is>
@@ -11160,7 +11190,7 @@
           <t>GIBB Benjamin</t>
         </is>
       </c>
-      <c r="U187" t="inlineStr">
+      <c r="X187" t="inlineStr">
         <is>
           <t>36711</t>
         </is>
@@ -11218,7 +11248,7 @@
           <t>BORGES Felipe</t>
         </is>
       </c>
-      <c r="U188" t="inlineStr">
+      <c r="X188" t="inlineStr">
         <is>
           <t>38012</t>
         </is>
@@ -11276,7 +11306,7 @@
           <t>JEGOU Liam</t>
         </is>
       </c>
-      <c r="U189" t="inlineStr">
+      <c r="X189" t="inlineStr">
         <is>
           <t>35820</t>
         </is>
@@ -11334,7 +11364,7 @@
           <t>COF Blaz</t>
         </is>
       </c>
-      <c r="U190" t="inlineStr">
+      <c r="X190" t="inlineStr">
         <is>
           <t>36897</t>
         </is>
@@ -11392,7 +11422,7 @@
           <t>MARINIC Matija</t>
         </is>
       </c>
-      <c r="U191" t="inlineStr">
+      <c r="X191" t="inlineStr">
         <is>
           <t>35595</t>
         </is>
@@ -11450,7 +11480,7 @@
           <t>BREUER Florian</t>
         </is>
       </c>
-      <c r="U192" t="inlineStr">
+      <c r="X192" t="inlineStr">
         <is>
           <t>39171</t>
         </is>
@@ -11508,7 +11538,7 @@
           <t>THOMAS Martin</t>
         </is>
       </c>
-      <c r="U193" t="inlineStr">
+      <c r="X193" t="inlineStr">
         <is>
           <t>35412</t>
         </is>
@@ -11566,7 +11596,7 @@
           <t>GEBAS Vitezslav</t>
         </is>
       </c>
-      <c r="U194" t="inlineStr">
+      <c r="X194" t="inlineStr">
         <is>
           <t>35038</t>
         </is>
@@ -11624,7 +11654,7 @@
           <t>ANTON Franz</t>
         </is>
       </c>
-      <c r="U195" t="inlineStr">
+      <c r="X195" t="inlineStr">
         <is>
           <t>35137</t>
         </is>
@@ -11682,7 +11712,7 @@
           <t>ZHANG Jinjie</t>
         </is>
       </c>
-      <c r="U196" t="inlineStr">
+      <c r="X196" t="inlineStr">
         <is>
           <t>72213</t>
         </is>
@@ -11740,7 +11770,7 @@
           <t>WALL Demelza</t>
         </is>
       </c>
-      <c r="U197" t="inlineStr">
+      <c r="X197" t="inlineStr">
         <is>
           <t>60107</t>
         </is>
@@ -11798,7 +11828,7 @@
           <t>O'FERRALL Caoimhe</t>
         </is>
       </c>
-      <c r="U198" t="inlineStr">
+      <c r="X198" t="inlineStr">
         <is>
           <t>61007</t>
         </is>
@@ -11856,7 +11886,7 @@
           <t>NOVAK Lea</t>
         </is>
       </c>
-      <c r="U199" t="inlineStr">
+      <c r="X199" t="inlineStr">
         <is>
           <t>60323</t>
         </is>
@@ -11914,7 +11944,7 @@
           <t>YAGI Airi</t>
         </is>
       </c>
-      <c r="U200" t="inlineStr">
+      <c r="X200" t="inlineStr">
         <is>
           <t>37756</t>
         </is>
@@ -11972,7 +12002,7 @@
           <t>BETTERIDGE Lois</t>
         </is>
       </c>
-      <c r="U201" t="inlineStr">
+      <c r="X201" t="inlineStr">
         <is>
           <t>60078</t>
         </is>
@@ -12030,7 +12060,7 @@
           <t>DUANGLAWA Atcharaporn</t>
         </is>
       </c>
-      <c r="U202" t="inlineStr">
+      <c r="X202" t="inlineStr">
         <is>
           <t>61799</t>
         </is>
@@ -12088,7 +12118,7 @@
           <t>SATO Ayano</t>
         </is>
       </c>
-      <c r="U203" t="inlineStr">
+      <c r="X203" t="inlineStr">
         <is>
           <t>60374</t>
         </is>
@@ -12199,7 +12229,7 @@
           <t>GLEJTEKOVA Simona</t>
         </is>
       </c>
-      <c r="U205" t="inlineStr">
+      <c r="X205" t="inlineStr">
         <is>
           <t>55166</t>
         </is>
@@ -12257,7 +12287,7 @@
           <t>MACEKOVA Simona</t>
         </is>
       </c>
-      <c r="U206" t="inlineStr">
+      <c r="X206" t="inlineStr">
         <is>
           <t>45153</t>
         </is>
@@ -12315,7 +12345,7 @@
           <t>BIZJAK Nina</t>
         </is>
       </c>
-      <c r="U207" t="inlineStr">
+      <c r="X207" t="inlineStr">
         <is>
           <t>39984</t>
         </is>
@@ -12373,7 +12403,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U208" t="inlineStr">
+      <c r="X208" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -12431,7 +12461,7 @@
           <t>JANCZY Justyna</t>
         </is>
       </c>
-      <c r="U209" t="inlineStr">
+      <c r="X209" t="inlineStr">
         <is>
           <t>43975</t>
         </is>
@@ -12489,7 +12519,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U210" t="inlineStr">
+      <c r="X210" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -12547,7 +12577,7 @@
           <t>MATULKOVA Jana</t>
         </is>
       </c>
-      <c r="U211" t="inlineStr">
+      <c r="X211" t="inlineStr">
         <is>
           <t>37274</t>
         </is>
@@ -12605,7 +12635,7 @@
           <t>PRIOUX Lucie</t>
         </is>
       </c>
-      <c r="U212" t="inlineStr">
+      <c r="X212" t="inlineStr">
         <is>
           <t>42984</t>
         </is>
@@ -12663,7 +12693,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U213" t="inlineStr">
+      <c r="X213" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -12721,7 +12751,7 @@
           <t>LAUNAY Damien</t>
         </is>
       </c>
-      <c r="U214" t="inlineStr">
+      <c r="X214" t="inlineStr">
         <is>
           <t>60047</t>
         </is>
@@ -12779,7 +12809,7 @@
           <t>SIMPSON Keenan</t>
         </is>
       </c>
-      <c r="U215" t="inlineStr">
+      <c r="X215" t="inlineStr">
         <is>
           <t>71797</t>
         </is>
@@ -12837,7 +12867,7 @@
           <t>MUSGRAVE Andrew</t>
         </is>
       </c>
-      <c r="U216" t="inlineStr">
+      <c r="X216" t="inlineStr">
         <is>
           <t>60102</t>
         </is>
@@ -12895,7 +12925,7 @@
           <t>HENDRICK Noel</t>
         </is>
       </c>
-      <c r="U217" t="inlineStr">
+      <c r="X217" t="inlineStr">
         <is>
           <t>43003</t>
         </is>
@@ -12953,7 +12983,7 @@
           <t>STOILJKOVIC Dusan</t>
         </is>
       </c>
-      <c r="U218" t="inlineStr">
+      <c r="X218" t="inlineStr">
         <is>
           <t>35791</t>
         </is>
@@ -13011,7 +13041,7 @@
           <t>BOWERS Christopher</t>
         </is>
       </c>
-      <c r="U219" t="inlineStr">
+      <c r="X219" t="inlineStr">
         <is>
           <t>52010</t>
         </is>
@@ -13069,7 +13099,7 @@
           <t>KORPES Ren</t>
         </is>
       </c>
-      <c r="U220" t="inlineStr">
+      <c r="X220" t="inlineStr">
         <is>
           <t>39941</t>
         </is>
@@ -13127,7 +13157,7 @@
           <t>SASAKI Tsubasa Terry</t>
         </is>
       </c>
-      <c r="U221" t="inlineStr">
+      <c r="X221" t="inlineStr">
         <is>
           <t>47085</t>
         </is>
@@ -13185,7 +13215,7 @@
           <t>MAIKRANZ Alexandr</t>
         </is>
       </c>
-      <c r="U222" t="inlineStr">
+      <c r="X222" t="inlineStr">
         <is>
           <t>60018</t>
         </is>
@@ -13243,7 +13273,7 @@
           <t>TRAVOSTINO Benjamin</t>
         </is>
       </c>
-      <c r="U223" t="inlineStr">
+      <c r="X223" t="inlineStr">
         <is>
           <t>68795</t>
         </is>
@@ -13301,7 +13331,7 @@
           <t>SANDERA Wiktor</t>
         </is>
       </c>
-      <c r="U224" t="inlineStr">
+      <c r="X224" t="inlineStr">
         <is>
           <t>53642</t>
         </is>
@@ -13359,7 +13389,7 @@
           <t>LEE EDWARDS Ciaran</t>
         </is>
       </c>
-      <c r="U225" t="inlineStr">
+      <c r="X225" t="inlineStr">
         <is>
           <t>35614</t>
         </is>
@@ -13417,7 +13447,7 @@
           <t>LLORENTE David</t>
         </is>
       </c>
-      <c r="U226" t="inlineStr">
+      <c r="X226" t="inlineStr">
         <is>
           <t>51850</t>
         </is>
@@ -13475,7 +13505,7 @@
           <t>CURTIS Samuel</t>
         </is>
       </c>
-      <c r="U227" t="inlineStr">
+      <c r="X227" t="inlineStr">
         <is>
           <t>36683</t>
         </is>
@@ -13533,7 +13563,7 @@
           <t>KANAYA Tohru</t>
         </is>
       </c>
-      <c r="U228" t="inlineStr">
+      <c r="X228" t="inlineStr">
         <is>
           <t>36484</t>
         </is>
@@ -13591,7 +13621,7 @@
           <t>POPE Benjamin</t>
         </is>
       </c>
-      <c r="U229" t="inlineStr">
+      <c r="X229" t="inlineStr">
         <is>
           <t>51753</t>
         </is>
@@ -13649,7 +13679,7 @@
           <t>MUNSCH Manuel</t>
         </is>
       </c>
-      <c r="U230" t="inlineStr">
+      <c r="X230" t="inlineStr">
         <is>
           <t>35631</t>
         </is>
@@ -13707,7 +13737,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U231" t="inlineStr">
+      <c r="X231" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -13765,7 +13795,7 @@
           <t>BEDA Marcello</t>
         </is>
       </c>
-      <c r="U232" t="inlineStr">
+      <c r="X232" t="inlineStr">
         <is>
           <t>39899</t>
         </is>
@@ -13823,7 +13853,7 @@
           <t>TAN Ya</t>
         </is>
       </c>
-      <c r="U233" t="inlineStr">
+      <c r="X233" t="inlineStr">
         <is>
           <t>52024</t>
         </is>
@@ -13881,7 +13911,7 @@
           <t>WEGER Matthias</t>
         </is>
       </c>
-      <c r="U234" t="inlineStr">
+      <c r="X234" t="inlineStr">
         <is>
           <t>68837</t>
         </is>
@@ -13939,7 +13969,7 @@
           <t>CADENA Jordi</t>
         </is>
       </c>
-      <c r="U235" t="inlineStr">
+      <c r="X235" t="inlineStr">
         <is>
           <t>41644</t>
         </is>
@@ -13997,7 +14027,7 @@
           <t>TAYLER Michael</t>
         </is>
       </c>
-      <c r="U236" t="inlineStr">
+      <c r="X236" t="inlineStr">
         <is>
           <t>36262</t>
         </is>
@@ -14055,7 +14085,7 @@
           <t>DOUGOUD Martin</t>
         </is>
       </c>
-      <c r="U237" t="inlineStr">
+      <c r="X237" t="inlineStr">
         <is>
           <t>35426</t>
         </is>
@@ -14166,7 +14196,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U239" t="inlineStr">
+      <c r="X239" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -14224,7 +14254,7 @@
           <t>POTOCNY Marcel</t>
         </is>
       </c>
-      <c r="U240" t="inlineStr">
+      <c r="X240" t="inlineStr">
         <is>
           <t>35235</t>
         </is>
@@ -14282,7 +14312,7 @@
           <t>HUJSA Matus</t>
         </is>
       </c>
-      <c r="U241" t="inlineStr">
+      <c r="X241" t="inlineStr">
         <is>
           <t>35503</t>
         </is>
@@ -14340,7 +14370,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U242" t="inlineStr">
+      <c r="X242" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -14451,7 +14481,7 @@
           <t>MALEK Andrej</t>
         </is>
       </c>
-      <c r="U244" t="inlineStr">
+      <c r="X244" t="inlineStr">
         <is>
           <t>39246</t>
         </is>
@@ -14509,7 +14539,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U245" t="inlineStr">
+      <c r="X245" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -14567,7 +14597,7 @@
           <t>BOURLIAUD Pierre</t>
         </is>
       </c>
-      <c r="U246" t="inlineStr">
+      <c r="X246" t="inlineStr">
         <is>
           <t>35230</t>
         </is>
@@ -14625,7 +14655,7 @@
           <t>GRIGAR Jakub</t>
         </is>
       </c>
-      <c r="U247" t="inlineStr">
+      <c r="X247" t="inlineStr">
         <is>
           <t>37284</t>
         </is>
@@ -14683,7 +14713,7 @@
           <t>NEVEU Boris</t>
         </is>
       </c>
-      <c r="U248" t="inlineStr">
+      <c r="X248" t="inlineStr">
         <is>
           <t>35396</t>
         </is>
@@ -14794,7 +14824,7 @@
           <t>BETTERIDGE Lois</t>
         </is>
       </c>
-      <c r="U250" t="inlineStr">
+      <c r="X250" t="inlineStr">
         <is>
           <t>60078</t>
         </is>
@@ -14852,7 +14882,7 @@
           <t>CHEN Shi</t>
         </is>
       </c>
-      <c r="U251" t="inlineStr">
+      <c r="X251" t="inlineStr">
         <is>
           <t>52027</t>
         </is>
@@ -14963,7 +14993,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U253" t="inlineStr">
+      <c r="X253" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -15021,7 +15051,7 @@
           <t>GUIET Pauline</t>
         </is>
       </c>
-      <c r="U254" t="inlineStr">
+      <c r="X254" t="inlineStr">
         <is>
           <t>35493</t>
         </is>
@@ -15079,7 +15109,7 @@
           <t>RANDLE Kensa</t>
         </is>
       </c>
-      <c r="U255" t="inlineStr">
+      <c r="X255" t="inlineStr">
         <is>
           <t>51859</t>
         </is>
@@ -15137,7 +15167,7 @@
           <t>OKAZAKI Haruka</t>
         </is>
       </c>
-      <c r="U256" t="inlineStr">
+      <c r="X256" t="inlineStr">
         <is>
           <t>42265</t>
         </is>
@@ -15195,7 +15225,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U257" t="inlineStr">
+      <c r="X257" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -15306,7 +15336,7 @@
           <t>MAHEU Florence</t>
         </is>
       </c>
-      <c r="U259" t="inlineStr">
+      <c r="X259" t="inlineStr">
         <is>
           <t>36416</t>
         </is>
@@ -15417,7 +15447,7 @@
           <t>HASSOVA Michaela</t>
         </is>
       </c>
-      <c r="U261" t="inlineStr">
+      <c r="X261" t="inlineStr">
         <is>
           <t>41783</t>
         </is>
@@ -15475,7 +15505,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U262" t="inlineStr">
+      <c r="X262" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -15533,7 +15563,7 @@
           <t>CWIK Sara</t>
         </is>
       </c>
-      <c r="U263" t="inlineStr">
+      <c r="X263" t="inlineStr">
         <is>
           <t>43978</t>
         </is>
@@ -15591,7 +15621,7 @@
           <t>TROMPETER Caroline</t>
         </is>
       </c>
-      <c r="U264" t="inlineStr">
+      <c r="X264" t="inlineStr">
         <is>
           <t>39167</t>
         </is>
@@ -15649,7 +15679,7 @@
           <t>GROENEVELD Jessica</t>
         </is>
       </c>
-      <c r="U265" t="inlineStr">
+      <c r="X265" t="inlineStr">
         <is>
           <t>35542</t>
         </is>
@@ -15760,7 +15790,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U267" t="inlineStr">
+      <c r="X267" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -15818,7 +15848,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U268" t="inlineStr">
+      <c r="X268" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -15876,7 +15906,7 @@
           <t>SABATTINI Chiara</t>
         </is>
       </c>
-      <c r="U269" t="inlineStr">
+      <c r="X269" t="inlineStr">
         <is>
           <t>35219</t>
         </is>
@@ -15934,7 +15964,7 @@
           <t>TAKESHITA Yuriko</t>
         </is>
       </c>
-      <c r="U270" t="inlineStr">
+      <c r="X270" t="inlineStr">
         <is>
           <t>36487</t>
         </is>
@@ -16045,7 +16075,7 @@
           <t>MEDON Joanna</t>
         </is>
       </c>
-      <c r="U272" t="inlineStr">
+      <c r="X272" t="inlineStr">
         <is>
           <t>35438</t>
         </is>
@@ -16156,7 +16186,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U274" t="inlineStr">
+      <c r="X274" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -16214,7 +16244,7 @@
           <t>WEGMAN Martina</t>
         </is>
       </c>
-      <c r="U275" t="inlineStr">
+      <c r="X275" t="inlineStr">
         <is>
           <t>35345</t>
         </is>
@@ -16272,7 +16302,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U276" t="inlineStr">
+      <c r="X276" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -16330,7 +16360,7 @@
           <t>KALISKA Elena</t>
         </is>
       </c>
-      <c r="U277" t="inlineStr">
+      <c r="X277" t="inlineStr">
         <is>
           <t>35366</t>
         </is>
@@ -16388,7 +16418,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U278" t="inlineStr">
+      <c r="X278" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -16446,7 +16476,7 @@
           <t>BOUZIDI Carole</t>
         </is>
       </c>
-      <c r="U279" t="inlineStr">
+      <c r="X279" t="inlineStr">
         <is>
           <t>35231</t>
         </is>
@@ -16504,7 +16534,7 @@
           <t>MANGIN Estelle</t>
         </is>
       </c>
-      <c r="U280" t="inlineStr">
+      <c r="X280" t="inlineStr">
         <is>
           <t>35670</t>
         </is>
@@ -16562,7 +16592,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U281" t="inlineStr">
+      <c r="X281" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -16620,7 +16650,7 @@
           <t>OBLINGER-PETERS Violetta</t>
         </is>
       </c>
-      <c r="U282" t="inlineStr">
+      <c r="X282" t="inlineStr">
         <is>
           <t>35289</t>
         </is>
@@ -16678,7 +16708,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U283" t="inlineStr">
+      <c r="X283" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -16736,7 +16766,7 @@
           <t>PENNIE Fiona</t>
         </is>
       </c>
-      <c r="U284" t="inlineStr">
+      <c r="X284" t="inlineStr">
         <is>
           <t>35638</t>
         </is>
@@ -16794,7 +16824,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U285" t="inlineStr">
+      <c r="X285" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -16905,7 +16935,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U287" t="inlineStr">
+      <c r="X287" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -16963,7 +16993,7 @@
           <t>MARTINEZ Marta</t>
         </is>
       </c>
-      <c r="U288" t="inlineStr">
+      <c r="X288" t="inlineStr">
         <is>
           <t>35760</t>
         </is>
@@ -17021,7 +17051,7 @@
           <t>KRAGELJ Ursa</t>
         </is>
       </c>
-      <c r="U289" t="inlineStr">
+      <c r="X289" t="inlineStr">
         <is>
           <t>36264</t>
         </is>
@@ -17079,7 +17109,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U290" t="inlineStr">
+      <c r="X290" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -17137,7 +17167,7 @@
           <t>DUKATOVA Jana</t>
         </is>
       </c>
-      <c r="U291" t="inlineStr">
+      <c r="X291" t="inlineStr">
         <is>
           <t>35354</t>
         </is>
@@ -17195,7 +17225,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U292" t="inlineStr">
+      <c r="X292" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -17253,7 +17283,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U293" t="inlineStr">
+      <c r="X293" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -17311,7 +17341,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U294" t="inlineStr">
+      <c r="X294" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -17374,12 +17404,12 @@
           <t>XIE Yuancong</t>
         </is>
       </c>
-      <c r="U295" t="inlineStr">
+      <c r="X295" t="inlineStr">
         <is>
           <t>42912</t>
         </is>
       </c>
-      <c r="V295" t="inlineStr">
+      <c r="Y295" t="inlineStr">
         <is>
           <t>72214</t>
         </is>
@@ -17442,12 +17472,12 @@
           <t>WEBER Alexander</t>
         </is>
       </c>
-      <c r="U296" t="inlineStr">
+      <c r="X296" t="inlineStr">
         <is>
           <t>51833</t>
         </is>
       </c>
-      <c r="V296" t="inlineStr">
+      <c r="Y296" t="inlineStr">
         <is>
           <t>51832</t>
         </is>
@@ -17510,12 +17540,12 @@
           <t>KASPAR Albert</t>
         </is>
       </c>
-      <c r="U297" t="inlineStr">
+      <c r="X297" t="inlineStr">
         <is>
           <t>42012</t>
         </is>
       </c>
-      <c r="V297" t="inlineStr">
+      <c r="Y297" t="inlineStr">
         <is>
           <t>42013</t>
         </is>
@@ -17578,12 +17608,12 @@
           <t>CHEN Jin</t>
         </is>
       </c>
-      <c r="U298" t="inlineStr">
+      <c r="X298" t="inlineStr">
         <is>
           <t>42237</t>
         </is>
       </c>
-      <c r="V298" t="inlineStr">
+      <c r="Y298" t="inlineStr">
         <is>
           <t>42238</t>
         </is>
@@ -17646,12 +17676,12 @@
           <t>DENG Xiao</t>
         </is>
       </c>
-      <c r="U299" t="inlineStr">
+      <c r="X299" t="inlineStr">
         <is>
           <t>42239</t>
         </is>
       </c>
-      <c r="V299" t="inlineStr">
+      <c r="Y299" t="inlineStr">
         <is>
           <t>42240</t>
         </is>
@@ -17714,12 +17744,12 @@
           <t>EICHFELD Casey</t>
         </is>
       </c>
-      <c r="U300" t="inlineStr">
+      <c r="X300" t="inlineStr">
         <is>
           <t>35068</t>
         </is>
       </c>
-      <c r="V300" t="inlineStr">
+      <c r="Y300" t="inlineStr">
         <is>
           <t>35067</t>
         </is>
@@ -17782,12 +17812,12 @@
           <t>OLIVEIRA Anderson</t>
         </is>
       </c>
-      <c r="U301" t="inlineStr">
+      <c r="X301" t="inlineStr">
         <is>
           <t>38018</t>
         </is>
       </c>
-      <c r="V301" t="inlineStr">
+      <c r="Y301" t="inlineStr">
         <is>
           <t>38020</t>
         </is>
@@ -17850,12 +17880,12 @@
           <t>WERRO Simon</t>
         </is>
       </c>
-      <c r="U302" t="inlineStr">
+      <c r="X302" t="inlineStr">
         <is>
           <t>35347</t>
         </is>
       </c>
-      <c r="V302" t="inlineStr">
+      <c r="Y302" t="inlineStr">
         <is>
           <t>35424</t>
         </is>
@@ -17918,12 +17948,12 @@
           <t>VRZAN Jakub</t>
         </is>
       </c>
-      <c r="U303" t="inlineStr">
+      <c r="X303" t="inlineStr">
         <is>
           <t>35042</t>
         </is>
       </c>
-      <c r="V303" t="inlineStr">
+      <c r="Y303" t="inlineStr">
         <is>
           <t>35043</t>
         </is>
@@ -17986,12 +18016,12 @@
           <t>MAJERCZAK Grzegorz</t>
         </is>
       </c>
-      <c r="U304" t="inlineStr">
+      <c r="X304" t="inlineStr">
         <is>
           <t>35085</t>
         </is>
       </c>
-      <c r="V304" t="inlineStr">
+      <c r="Y304" t="inlineStr">
         <is>
           <t>35086</t>
         </is>
@@ -18054,12 +18084,12 @@
           <t>BRZEZINSKI Andrzej</t>
         </is>
       </c>
-      <c r="U305" t="inlineStr">
+      <c r="X305" t="inlineStr">
         <is>
           <t>35082</t>
         </is>
       </c>
-      <c r="V305" t="inlineStr">
+      <c r="Y305" t="inlineStr">
         <is>
           <t>35081</t>
         </is>
@@ -18122,12 +18152,12 @@
           <t>MUELLER Kevin</t>
         </is>
       </c>
-      <c r="U306" t="inlineStr">
+      <c r="X306" t="inlineStr">
         <is>
           <t>35148</t>
         </is>
       </c>
-      <c r="V306" t="inlineStr">
+      <c r="Y306" t="inlineStr">
         <is>
           <t>35149</t>
         </is>
@@ -18190,12 +18220,12 @@
           <t>BETTGE Nico</t>
         </is>
       </c>
-      <c r="U307" t="inlineStr">
+      <c r="X307" t="inlineStr">
         <is>
           <t>35145</t>
         </is>
       </c>
-      <c r="V307" t="inlineStr">
+      <c r="Y307" t="inlineStr">
         <is>
           <t>35133</t>
         </is>
@@ -18258,12 +18288,12 @@
           <t>BATIK Jan</t>
         </is>
       </c>
-      <c r="U308" t="inlineStr">
+      <c r="X308" t="inlineStr">
         <is>
           <t>35368</t>
         </is>
       </c>
-      <c r="V308" t="inlineStr">
+      <c r="Y308" t="inlineStr">
         <is>
           <t>35367</t>
         </is>
@@ -18326,12 +18356,12 @@
           <t>CAILHOL Hugo</t>
         </is>
       </c>
-      <c r="U309" t="inlineStr">
+      <c r="X309" t="inlineStr">
         <is>
           <t>35476</t>
         </is>
       </c>
-      <c r="V309" t="inlineStr">
+      <c r="Y309" t="inlineStr">
         <is>
           <t>35491</t>
         </is>
@@ -18394,12 +18424,12 @@
           <t>LE RUYET Edern</t>
         </is>
       </c>
-      <c r="U310" t="inlineStr">
+      <c r="X310" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
       </c>
-      <c r="V310" t="inlineStr">
+      <c r="Y310" t="inlineStr">
         <is>
           <t>35379</t>
         </is>
@@ -18462,12 +18492,12 @@
           <t>POCHWALA Marcin</t>
         </is>
       </c>
-      <c r="U311" t="inlineStr">
+      <c r="X311" t="inlineStr">
         <is>
           <t>35080</t>
         </is>
       </c>
-      <c r="V311" t="inlineStr">
+      <c r="Y311" t="inlineStr">
         <is>
           <t>35079</t>
         </is>
@@ -18530,12 +18560,12 @@
           <t>JANE Jakub</t>
         </is>
       </c>
-      <c r="U312" t="inlineStr">
+      <c r="X312" t="inlineStr">
         <is>
           <t>35060</t>
         </is>
       </c>
-      <c r="V312" t="inlineStr">
+      <c r="Y312" t="inlineStr">
         <is>
           <t>35061</t>
         </is>
@@ -18598,12 +18628,12 @@
           <t>TALJAT Saso</t>
         </is>
       </c>
-      <c r="U313" t="inlineStr">
+      <c r="X313" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
       </c>
-      <c r="V313" t="inlineStr">
+      <c r="Y313" t="inlineStr">
         <is>
           <t>36270</t>
         </is>
@@ -18666,12 +18696,12 @@
           <t>BECKER Thomas</t>
         </is>
       </c>
-      <c r="U314" t="inlineStr">
+      <c r="X314" t="inlineStr">
         <is>
           <t>35139</t>
         </is>
       </c>
-      <c r="V314" t="inlineStr">
+      <c r="Y314" t="inlineStr">
         <is>
           <t>35143</t>
         </is>
@@ -18734,12 +18764,12 @@
           <t>BISO Hugo</t>
         </is>
       </c>
-      <c r="U315" t="inlineStr">
+      <c r="X315" t="inlineStr">
         <is>
           <t>35403</t>
         </is>
       </c>
-      <c r="V315" t="inlineStr">
+      <c r="Y315" t="inlineStr">
         <is>
           <t>35229</t>
         </is>
@@ -18802,12 +18832,12 @@
           <t>SKANTAR Peter</t>
         </is>
       </c>
-      <c r="U316" t="inlineStr">
+      <c r="X316" t="inlineStr">
         <is>
           <t>35360</t>
         </is>
       </c>
-      <c r="V316" t="inlineStr">
+      <c r="Y316" t="inlineStr">
         <is>
           <t>35361</t>
         </is>
@@ -18918,7 +18948,7 @@
           <t>BETTERIDGE Lois</t>
         </is>
       </c>
-      <c r="U318" t="inlineStr">
+      <c r="X318" t="inlineStr">
         <is>
           <t>60078</t>
         </is>
@@ -18976,7 +19006,7 @@
           <t>CHEN Shi</t>
         </is>
       </c>
-      <c r="U319" t="inlineStr">
+      <c r="X319" t="inlineStr">
         <is>
           <t>52027</t>
         </is>
@@ -19087,7 +19117,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U321" t="inlineStr">
+      <c r="X321" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -19145,7 +19175,7 @@
           <t>RANDLE Kensa</t>
         </is>
       </c>
-      <c r="U322" t="inlineStr">
+      <c r="X322" t="inlineStr">
         <is>
           <t>51859</t>
         </is>
@@ -19203,7 +19233,7 @@
           <t>OKAZAKI Haruka</t>
         </is>
       </c>
-      <c r="U323" t="inlineStr">
+      <c r="X323" t="inlineStr">
         <is>
           <t>42265</t>
         </is>
@@ -19261,7 +19291,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U324" t="inlineStr">
+      <c r="X324" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -19372,7 +19402,7 @@
           <t>MAHEU Florence</t>
         </is>
       </c>
-      <c r="U326" t="inlineStr">
+      <c r="X326" t="inlineStr">
         <is>
           <t>36416</t>
         </is>
@@ -19483,7 +19513,7 @@
           <t>HASSOVA Michaela</t>
         </is>
       </c>
-      <c r="U328" t="inlineStr">
+      <c r="X328" t="inlineStr">
         <is>
           <t>41783</t>
         </is>
@@ -19541,7 +19571,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U329" t="inlineStr">
+      <c r="X329" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -19599,7 +19629,7 @@
           <t>CWIK Sara</t>
         </is>
       </c>
-      <c r="U330" t="inlineStr">
+      <c r="X330" t="inlineStr">
         <is>
           <t>43978</t>
         </is>
@@ -19657,7 +19687,7 @@
           <t>GROENEVELD Jessica</t>
         </is>
       </c>
-      <c r="U331" t="inlineStr">
+      <c r="X331" t="inlineStr">
         <is>
           <t>35542</t>
         </is>
@@ -19768,7 +19798,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U333" t="inlineStr">
+      <c r="X333" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -19826,7 +19856,7 @@
           <t>SABATTINI Chiara</t>
         </is>
       </c>
-      <c r="U334" t="inlineStr">
+      <c r="X334" t="inlineStr">
         <is>
           <t>35219</t>
         </is>
@@ -19884,7 +19914,7 @@
           <t>TAKESHITA Yuriko</t>
         </is>
       </c>
-      <c r="U335" t="inlineStr">
+      <c r="X335" t="inlineStr">
         <is>
           <t>36487</t>
         </is>
@@ -19995,7 +20025,7 @@
           <t>MEDON Joanna</t>
         </is>
       </c>
-      <c r="U337" t="inlineStr">
+      <c r="X337" t="inlineStr">
         <is>
           <t>35438</t>
         </is>
@@ -20106,7 +20136,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U339" t="inlineStr">
+      <c r="X339" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -20164,7 +20194,7 @@
           <t>WEGMAN Martina</t>
         </is>
       </c>
-      <c r="U340" t="inlineStr">
+      <c r="X340" t="inlineStr">
         <is>
           <t>35345</t>
         </is>
@@ -20222,7 +20252,7 @@
           <t>KALISKA Elena</t>
         </is>
       </c>
-      <c r="U341" t="inlineStr">
+      <c r="X341" t="inlineStr">
         <is>
           <t>35366</t>
         </is>
@@ -20280,7 +20310,7 @@
           <t>KRAGELJ Ursa</t>
         </is>
       </c>
-      <c r="U342" t="inlineStr">
+      <c r="X342" t="inlineStr">
         <is>
           <t>36264</t>
         </is>
@@ -20343,12 +20373,12 @@
           <t>XIE Yuancong</t>
         </is>
       </c>
-      <c r="U343" t="inlineStr">
+      <c r="X343" t="inlineStr">
         <is>
           <t>42912</t>
         </is>
       </c>
-      <c r="V343" t="inlineStr">
+      <c r="Y343" t="inlineStr">
         <is>
           <t>72214</t>
         </is>
@@ -20411,12 +20441,12 @@
           <t>WEBER Alexander</t>
         </is>
       </c>
-      <c r="U344" t="inlineStr">
+      <c r="X344" t="inlineStr">
         <is>
           <t>51833</t>
         </is>
       </c>
-      <c r="V344" t="inlineStr">
+      <c r="Y344" t="inlineStr">
         <is>
           <t>51832</t>
         </is>
@@ -20479,12 +20509,12 @@
           <t>KASPAR Albert</t>
         </is>
       </c>
-      <c r="U345" t="inlineStr">
+      <c r="X345" t="inlineStr">
         <is>
           <t>42012</t>
         </is>
       </c>
-      <c r="V345" t="inlineStr">
+      <c r="Y345" t="inlineStr">
         <is>
           <t>42013</t>
         </is>
@@ -20547,12 +20577,12 @@
           <t>DENG Xiao</t>
         </is>
       </c>
-      <c r="U346" t="inlineStr">
+      <c r="X346" t="inlineStr">
         <is>
           <t>42239</t>
         </is>
       </c>
-      <c r="V346" t="inlineStr">
+      <c r="Y346" t="inlineStr">
         <is>
           <t>42240</t>
         </is>
@@ -20615,12 +20645,12 @@
           <t>BETTGE Nico</t>
         </is>
       </c>
-      <c r="U347" t="inlineStr">
+      <c r="X347" t="inlineStr">
         <is>
           <t>35145</t>
         </is>
       </c>
-      <c r="V347" t="inlineStr">
+      <c r="Y347" t="inlineStr">
         <is>
           <t>35133</t>
         </is>
@@ -20683,12 +20713,12 @@
           <t>BATIK Jan</t>
         </is>
       </c>
-      <c r="U348" t="inlineStr">
+      <c r="X348" t="inlineStr">
         <is>
           <t>35368</t>
         </is>
       </c>
-      <c r="V348" t="inlineStr">
+      <c r="Y348" t="inlineStr">
         <is>
           <t>35367</t>
         </is>
@@ -20751,12 +20781,12 @@
           <t>JANE Jakub</t>
         </is>
       </c>
-      <c r="U349" t="inlineStr">
+      <c r="X349" t="inlineStr">
         <is>
           <t>35060</t>
         </is>
       </c>
-      <c r="V349" t="inlineStr">
+      <c r="Y349" t="inlineStr">
         <is>
           <t>35061</t>
         </is>
@@ -20915,7 +20945,7 @@
           <t>NOVAK Lea</t>
         </is>
       </c>
-      <c r="U352" t="inlineStr">
+      <c r="X352" t="inlineStr">
         <is>
           <t>60323</t>
         </is>
@@ -20973,7 +21003,7 @@
           <t>JANCZY Justyna</t>
         </is>
       </c>
-      <c r="U353" t="inlineStr">
+      <c r="X353" t="inlineStr">
         <is>
           <t>43975</t>
         </is>
@@ -21137,7 +21167,7 @@
           <t>JEGOU Liam</t>
         </is>
       </c>
-      <c r="U356" t="inlineStr">
+      <c r="X356" t="inlineStr">
         <is>
           <t>35820</t>
         </is>
@@ -21195,7 +21225,7 @@
           <t>MARINIC Matija</t>
         </is>
       </c>
-      <c r="U357" t="inlineStr">
+      <c r="X357" t="inlineStr">
         <is>
           <t>35595</t>
         </is>
@@ -21253,7 +21283,7 @@
           <t>TRAVE Miquel</t>
         </is>
       </c>
-      <c r="U358" t="inlineStr">
+      <c r="X358" t="inlineStr">
         <is>
           <t>68998</t>
         </is>
@@ -21311,7 +21341,7 @@
           <t>BORGES Felipe</t>
         </is>
       </c>
-      <c r="U359" t="inlineStr">
+      <c r="X359" t="inlineStr">
         <is>
           <t>38012</t>
         </is>
@@ -21369,7 +21399,7 @@
           <t>GEBAS Vitezslav</t>
         </is>
       </c>
-      <c r="U360" t="inlineStr">
+      <c r="X360" t="inlineStr">
         <is>
           <t>35038</t>
         </is>
@@ -21427,7 +21457,7 @@
           <t>THOMAS Martin</t>
         </is>
       </c>
-      <c r="U361" t="inlineStr">
+      <c r="X361" t="inlineStr">
         <is>
           <t>35412</t>
         </is>
@@ -21485,7 +21515,7 @@
           <t>COF Blaz</t>
         </is>
       </c>
-      <c r="U362" t="inlineStr">
+      <c r="X362" t="inlineStr">
         <is>
           <t>36897</t>
         </is>
@@ -21596,7 +21626,7 @@
           <t>BREUER Florian</t>
         </is>
       </c>
-      <c r="U364" t="inlineStr">
+      <c r="X364" t="inlineStr">
         <is>
           <t>39171</t>
         </is>
@@ -21654,7 +21684,7 @@
           <t>ANTON Franz</t>
         </is>
       </c>
-      <c r="U365" t="inlineStr">
+      <c r="X365" t="inlineStr">
         <is>
           <t>35137</t>
         </is>
@@ -21712,7 +21742,7 @@
           <t>BURGESS Adam</t>
         </is>
       </c>
-      <c r="U366" t="inlineStr">
+      <c r="X366" t="inlineStr">
         <is>
           <t>35647</t>
         </is>
@@ -21770,7 +21800,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U367" t="inlineStr">
+      <c r="X367" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -21828,7 +21858,7 @@
           <t>CECCON Paolo</t>
         </is>
       </c>
-      <c r="U368" t="inlineStr">
+      <c r="X368" t="inlineStr">
         <is>
           <t>39903</t>
         </is>
@@ -21886,7 +21916,7 @@
           <t>KOECHLIN Thomas</t>
         </is>
       </c>
-      <c r="U369" t="inlineStr">
+      <c r="X369" t="inlineStr">
         <is>
           <t>35419</t>
         </is>
@@ -21944,7 +21974,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U370" t="inlineStr">
+      <c r="X370" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -22002,7 +22032,7 @@
           <t>HEDWIG Grzegorz</t>
         </is>
       </c>
-      <c r="U371" t="inlineStr">
+      <c r="X371" t="inlineStr">
         <is>
           <t>35465</t>
         </is>
@@ -22060,7 +22090,7 @@
           <t>IVALDI Raffaello</t>
         </is>
       </c>
-      <c r="U372" t="inlineStr">
+      <c r="X372" t="inlineStr">
         <is>
           <t>35227</t>
         </is>
@@ -22118,7 +22148,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U373" t="inlineStr">
+      <c r="X373" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -22176,7 +22206,7 @@
           <t>COLAZINGARI Roberto</t>
         </is>
       </c>
-      <c r="U374" t="inlineStr">
+      <c r="X374" t="inlineStr">
         <is>
           <t>35223</t>
         </is>
@@ -22234,7 +22264,7 @@
           <t>BADURA Jergus</t>
         </is>
       </c>
-      <c r="U375" t="inlineStr">
+      <c r="X375" t="inlineStr">
         <is>
           <t>68767</t>
         </is>
@@ -22292,7 +22322,7 @@
           <t>WESTLEY Ryan</t>
         </is>
       </c>
-      <c r="U376" t="inlineStr">
+      <c r="X376" t="inlineStr">
         <is>
           <t>35651</t>
         </is>
@@ -22350,7 +22380,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U377" t="inlineStr">
+      <c r="X377" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -22408,7 +22438,7 @@
           <t>BERCIC Anze</t>
         </is>
       </c>
-      <c r="U378" t="inlineStr">
+      <c r="X378" t="inlineStr">
         <is>
           <t>36253</t>
         </is>
@@ -22466,7 +22496,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U379" t="inlineStr">
+      <c r="X379" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -22524,7 +22554,7 @@
           <t>BETTGE Nico</t>
         </is>
       </c>
-      <c r="U380" t="inlineStr">
+      <c r="X380" t="inlineStr">
         <is>
           <t>35133</t>
         </is>
@@ -22582,7 +22612,7 @@
           <t>LENARCIC Jure</t>
         </is>
       </c>
-      <c r="U381" t="inlineStr">
+      <c r="X381" t="inlineStr">
         <is>
           <t>36259</t>
         </is>
@@ -22640,7 +22670,7 @@
           <t>TILLARD Pierre-Antoine</t>
         </is>
       </c>
-      <c r="U382" t="inlineStr">
+      <c r="X382" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
@@ -22698,7 +22728,7 @@
           <t>PESCHIER Nicolas</t>
         </is>
       </c>
-      <c r="U383" t="inlineStr">
+      <c r="X383" t="inlineStr">
         <is>
           <t>35401</t>
         </is>
@@ -22756,7 +22786,7 @@
           <t>EICHFELD Casey</t>
         </is>
       </c>
-      <c r="U384" t="inlineStr">
+      <c r="X384" t="inlineStr">
         <is>
           <t>35067</t>
         </is>
@@ -22814,7 +22844,7 @@
           <t>BENUS Matej</t>
         </is>
       </c>
-      <c r="U385" t="inlineStr">
+      <c r="X385" t="inlineStr">
         <is>
           <t>35353</t>
         </is>
@@ -22872,7 +22902,7 @@
           <t>HUJSA Matus</t>
         </is>
       </c>
-      <c r="U386" t="inlineStr">
+      <c r="X386" t="inlineStr">
         <is>
           <t>35503</t>
         </is>
@@ -22930,7 +22960,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U387" t="inlineStr">
+      <c r="X387" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -22988,7 +23018,7 @@
           <t>WEGER Matthias</t>
         </is>
       </c>
-      <c r="U388" t="inlineStr">
+      <c r="X388" t="inlineStr">
         <is>
           <t>68837</t>
         </is>
@@ -23046,7 +23076,7 @@
           <t>POTOCNY Marcel</t>
         </is>
       </c>
-      <c r="U389" t="inlineStr">
+      <c r="X389" t="inlineStr">
         <is>
           <t>35235</t>
         </is>
@@ -23104,7 +23134,7 @@
           <t>BOWERS Christopher</t>
         </is>
       </c>
-      <c r="U390" t="inlineStr">
+      <c r="X390" t="inlineStr">
         <is>
           <t>52010</t>
         </is>
@@ -23162,7 +23192,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U391" t="inlineStr">
+      <c r="X391" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -23273,7 +23303,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U393" t="inlineStr">
+      <c r="X393" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -23331,7 +23361,7 @@
           <t>LLORENTE David</t>
         </is>
       </c>
-      <c r="U394" t="inlineStr">
+      <c r="X394" t="inlineStr">
         <is>
           <t>51850</t>
         </is>
@@ -23389,7 +23419,7 @@
           <t>NEVEU Boris</t>
         </is>
       </c>
-      <c r="U395" t="inlineStr">
+      <c r="X395" t="inlineStr">
         <is>
           <t>35396</t>
         </is>
@@ -23447,7 +23477,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U396" t="inlineStr">
+      <c r="X396" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -23505,7 +23535,7 @@
           <t>MAXEINER Tim</t>
         </is>
       </c>
-      <c r="U397" t="inlineStr">
+      <c r="X397" t="inlineStr">
         <is>
           <t>35117</t>
         </is>
@@ -23563,7 +23593,7 @@
           <t>BOECKELMANN Paul</t>
         </is>
       </c>
-      <c r="U398" t="inlineStr">
+      <c r="X398" t="inlineStr">
         <is>
           <t>35118</t>
         </is>
@@ -23621,7 +23651,7 @@
           <t>ADACHI Kazuya</t>
         </is>
       </c>
-      <c r="U399" t="inlineStr">
+      <c r="X399" t="inlineStr">
         <is>
           <t>36646</t>
         </is>
@@ -23679,7 +23709,7 @@
           <t>OSCHMAUTZ Felix</t>
         </is>
       </c>
-      <c r="U400" t="inlineStr">
+      <c r="X400" t="inlineStr">
         <is>
           <t>51856</t>
         </is>
@@ -23737,7 +23767,7 @@
           <t>HOLMER Erik</t>
         </is>
       </c>
-      <c r="U401" t="inlineStr">
+      <c r="X401" t="inlineStr">
         <is>
           <t>35104</t>
         </is>
@@ -23795,7 +23825,7 @@
           <t>BERSINGER Thomas</t>
         </is>
       </c>
-      <c r="U402" t="inlineStr">
+      <c r="X402" t="inlineStr">
         <is>
           <t>35228</t>
         </is>
@@ -23853,7 +23883,7 @@
           <t>TUNKA Ondrej</t>
         </is>
       </c>
-      <c r="U403" t="inlineStr">
+      <c r="X403" t="inlineStr">
         <is>
           <t>35947</t>
         </is>
@@ -23911,7 +23941,7 @@
           <t>FORBES-CRYANS Bradley</t>
         </is>
       </c>
-      <c r="U404" t="inlineStr">
+      <c r="X404" t="inlineStr">
         <is>
           <t>36513</t>
         </is>
@@ -23969,7 +23999,7 @@
           <t>POLACZYK Mateusz</t>
         </is>
       </c>
-      <c r="U405" t="inlineStr">
+      <c r="X405" t="inlineStr">
         <is>
           <t>35072</t>
         </is>
@@ -24027,7 +24057,7 @@
           <t>PETERLIN Janos</t>
         </is>
       </c>
-      <c r="U406" t="inlineStr">
+      <c r="X406" t="inlineStr">
         <is>
           <t>36268</t>
         </is>
@@ -24085,7 +24115,7 @@
           <t>WATKINS Daniel</t>
         </is>
       </c>
-      <c r="U407" t="inlineStr">
+      <c r="X407" t="inlineStr">
         <is>
           <t>38430</t>
         </is>
@@ -24143,7 +24173,7 @@
           <t>SRABOTNIK Martin</t>
         </is>
       </c>
-      <c r="U408" t="inlineStr">
+      <c r="X408" t="inlineStr">
         <is>
           <t>39080</t>
         </is>
@@ -24201,7 +24231,7 @@
           <t>BIAZIZZO Mathieu</t>
         </is>
       </c>
-      <c r="U409" t="inlineStr">
+      <c r="X409" t="inlineStr">
         <is>
           <t>35484</t>
         </is>
@@ -24259,7 +24289,7 @@
           <t>BUTCHER Finn</t>
         </is>
       </c>
-      <c r="U410" t="inlineStr">
+      <c r="X410" t="inlineStr">
         <is>
           <t>36663</t>
         </is>
@@ -24317,7 +24347,7 @@
           <t>DAILLE Etienne</t>
         </is>
       </c>
-      <c r="U411" t="inlineStr">
+      <c r="X411" t="inlineStr">
         <is>
           <t>35308</t>
         </is>
@@ -24375,7 +24405,7 @@
           <t>GRIMM Alexander</t>
         </is>
       </c>
-      <c r="U412" t="inlineStr">
+      <c r="X412" t="inlineStr">
         <is>
           <t>35112</t>
         </is>
@@ -24433,7 +24463,7 @@
           <t>OKREGLAK Maciej</t>
         </is>
       </c>
-      <c r="U413" t="inlineStr">
+      <c r="X413" t="inlineStr">
         <is>
           <t>35088</t>
         </is>
@@ -24491,7 +24521,7 @@
           <t>ANDERSON Timothy</t>
         </is>
       </c>
-      <c r="U414" t="inlineStr">
+      <c r="X414" t="inlineStr">
         <is>
           <t>38432</t>
         </is>
@@ -24549,7 +24579,7 @@
           <t>MEGLIC Jure</t>
         </is>
       </c>
-      <c r="U415" t="inlineStr">
+      <c r="X415" t="inlineStr">
         <is>
           <t>35590</t>
         </is>
@@ -24607,7 +24637,7 @@
           <t>HERNANZ Samuel</t>
         </is>
       </c>
-      <c r="U416" t="inlineStr">
+      <c r="X416" t="inlineStr">
         <is>
           <t>35786</t>
         </is>
@@ -24665,7 +24695,7 @@
           <t>POPIELA Dariusz</t>
         </is>
       </c>
-      <c r="U417" t="inlineStr">
+      <c r="X417" t="inlineStr">
         <is>
           <t>35096</t>
         </is>
@@ -24723,7 +24753,7 @@
           <t>HILGERT Lubos</t>
         </is>
       </c>
-      <c r="U418" t="inlineStr">
+      <c r="X418" t="inlineStr">
         <is>
           <t>35032</t>
         </is>
@@ -24781,7 +24811,7 @@
           <t>ALBREHT Martin</t>
         </is>
       </c>
-      <c r="U419" t="inlineStr">
+      <c r="X419" t="inlineStr">
         <is>
           <t>36898</t>
         </is>
@@ -24839,7 +24869,7 @@
           <t>IVALDI Zeno</t>
         </is>
       </c>
-      <c r="U420" t="inlineStr">
+      <c r="X420" t="inlineStr">
         <is>
           <t>35480</t>
         </is>
@@ -24897,7 +24927,7 @@
           <t>DE GENNARO Giovanni</t>
         </is>
       </c>
-      <c r="U421" t="inlineStr">
+      <c r="X421" t="inlineStr">
         <is>
           <t>35244</t>
         </is>
@@ -24955,7 +24985,7 @@
           <t>SCHUBERT Sebastian</t>
         </is>
       </c>
-      <c r="U422" t="inlineStr">
+      <c r="X422" t="inlineStr">
         <is>
           <t>35114</t>
         </is>
@@ -25013,7 +25043,7 @@
           <t>PRINDIS Vit</t>
         </is>
       </c>
-      <c r="U423" t="inlineStr">
+      <c r="X423" t="inlineStr">
         <is>
           <t>35065</t>
         </is>
@@ -25071,7 +25101,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U424" t="inlineStr">
+      <c r="X424" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -25129,7 +25159,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U425" t="inlineStr">
+      <c r="X425" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -25187,7 +25217,7 @@
           <t>BIZJAK Nina</t>
         </is>
       </c>
-      <c r="U426" t="inlineStr">
+      <c r="X426" t="inlineStr">
         <is>
           <t>39984</t>
         </is>
@@ -25245,7 +25275,7 @@
           <t>GLEJTEKOVA Simona</t>
         </is>
       </c>
-      <c r="U427" t="inlineStr">
+      <c r="X427" t="inlineStr">
         <is>
           <t>55166</t>
         </is>
@@ -25303,7 +25333,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U428" t="inlineStr">
+      <c r="X428" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -25361,7 +25391,7 @@
           <t>PRIOUX Lucie</t>
         </is>
       </c>
-      <c r="U429" t="inlineStr">
+      <c r="X429" t="inlineStr">
         <is>
           <t>42984</t>
         </is>
@@ -25419,7 +25449,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U430" t="inlineStr">
+      <c r="X430" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -25477,7 +25507,7 @@
           <t>NAVEAU Laurine</t>
         </is>
       </c>
-      <c r="U431" t="inlineStr">
+      <c r="X431" t="inlineStr">
         <is>
           <t>53246</t>
         </is>
@@ -25535,7 +25565,7 @@
           <t>WERATSCHNIG Nadine</t>
         </is>
       </c>
-      <c r="U432" t="inlineStr">
+      <c r="X432" t="inlineStr">
         <is>
           <t>41613</t>
         </is>
@@ -25593,7 +25623,7 @@
           <t>TIXIER Cecile</t>
         </is>
       </c>
-      <c r="U433" t="inlineStr">
+      <c r="X433" t="inlineStr">
         <is>
           <t>35687</t>
         </is>
@@ -25651,7 +25681,7 @@
           <t>GIBSON Eilidh</t>
         </is>
       </c>
-      <c r="U434" t="inlineStr">
+      <c r="X434" t="inlineStr">
         <is>
           <t>36708</t>
         </is>
@@ -25762,7 +25792,7 @@
           <t>KOZOROG Alja</t>
         </is>
       </c>
-      <c r="U436" t="inlineStr">
+      <c r="X436" t="inlineStr">
         <is>
           <t>39986</t>
         </is>
@@ -25820,7 +25850,7 @@
           <t>STANOVSKA Sona</t>
         </is>
       </c>
-      <c r="U437" t="inlineStr">
+      <c r="X437" t="inlineStr">
         <is>
           <t>51647</t>
         </is>
@@ -25878,7 +25908,7 @@
           <t>JACQUET Claire</t>
         </is>
       </c>
-      <c r="U438" t="inlineStr">
+      <c r="X438" t="inlineStr">
         <is>
           <t>35684</t>
         </is>
@@ -25936,7 +25966,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U439" t="inlineStr">
+      <c r="X439" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -25994,7 +26024,7 @@
           <t>VAN DER KNIJFF Annebel</t>
         </is>
       </c>
-      <c r="U440" t="inlineStr">
+      <c r="X440" t="inlineStr">
         <is>
           <t>39945</t>
         </is>
@@ -26158,7 +26188,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U443" t="inlineStr">
+      <c r="X443" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -26216,7 +26246,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U444" t="inlineStr">
+      <c r="X444" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -26274,7 +26304,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U445" t="inlineStr">
+      <c r="X445" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -26342,7 +26372,7 @@
           <t>BETTGE Nico</t>
         </is>
       </c>
-      <c r="U446" t="inlineStr">
+      <c r="X446" t="inlineStr">
         <is>
           <t>35133</t>
         </is>
@@ -26410,7 +26440,7 @@
           <t>LENARCIC Jure</t>
         </is>
       </c>
-      <c r="U447" t="inlineStr">
+      <c r="X447" t="inlineStr">
         <is>
           <t>36259</t>
         </is>
@@ -26478,7 +26508,7 @@
           <t>TILLARD Pierre-Antoine</t>
         </is>
       </c>
-      <c r="U448" t="inlineStr">
+      <c r="X448" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
@@ -26546,7 +26576,7 @@
           <t>PESCHIER Nicolas</t>
         </is>
       </c>
-      <c r="U449" t="inlineStr">
+      <c r="X449" t="inlineStr">
         <is>
           <t>35401</t>
         </is>
@@ -26614,7 +26644,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U450" t="inlineStr">
+      <c r="X450" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -26682,7 +26712,7 @@
           <t>COF Blaz</t>
         </is>
       </c>
-      <c r="U451" t="inlineStr">
+      <c r="X451" t="inlineStr">
         <is>
           <t>36897</t>
         </is>
@@ -26750,7 +26780,7 @@
           <t>BREUER Florian</t>
         </is>
       </c>
-      <c r="U452" t="inlineStr">
+      <c r="X452" t="inlineStr">
         <is>
           <t>39171</t>
         </is>
@@ -26818,7 +26848,7 @@
           <t>WESTLEY Ryan</t>
         </is>
       </c>
-      <c r="U453" t="inlineStr">
+      <c r="X453" t="inlineStr">
         <is>
           <t>35651</t>
         </is>
@@ -26886,7 +26916,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U454" t="inlineStr">
+      <c r="X454" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -26954,7 +26984,7 @@
           <t>BENUS Matej</t>
         </is>
       </c>
-      <c r="U455" t="inlineStr">
+      <c r="X455" t="inlineStr">
         <is>
           <t>35353</t>
         </is>
@@ -27022,7 +27052,7 @@
           <t>BURGESS Adam</t>
         </is>
       </c>
-      <c r="U456" t="inlineStr">
+      <c r="X456" t="inlineStr">
         <is>
           <t>35647</t>
         </is>
@@ -27090,7 +27120,7 @@
           <t>KOECHLIN Thomas</t>
         </is>
       </c>
-      <c r="U457" t="inlineStr">
+      <c r="X457" t="inlineStr">
         <is>
           <t>35419</t>
         </is>
@@ -27158,7 +27188,7 @@
           <t>HEDWIG Grzegorz</t>
         </is>
       </c>
-      <c r="U458" t="inlineStr">
+      <c r="X458" t="inlineStr">
         <is>
           <t>35465</t>
         </is>
@@ -27226,7 +27256,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U459" t="inlineStr">
+      <c r="X459" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -27294,7 +27324,7 @@
           <t>EICHFELD Casey</t>
         </is>
       </c>
-      <c r="U460" t="inlineStr">
+      <c r="X460" t="inlineStr">
         <is>
           <t>35067</t>
         </is>
@@ -27362,7 +27392,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U461" t="inlineStr">
+      <c r="X461" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -27430,7 +27460,7 @@
           <t>BIAZIZZO Mathieu</t>
         </is>
       </c>
-      <c r="U462" t="inlineStr">
+      <c r="X462" t="inlineStr">
         <is>
           <t>35484</t>
         </is>
@@ -27498,7 +27528,7 @@
           <t>ADACHI Kazuya</t>
         </is>
       </c>
-      <c r="U463" t="inlineStr">
+      <c r="X463" t="inlineStr">
         <is>
           <t>36646</t>
         </is>
@@ -27566,7 +27596,7 @@
           <t>FORBES-CRYANS Bradley</t>
         </is>
       </c>
-      <c r="U464" t="inlineStr">
+      <c r="X464" t="inlineStr">
         <is>
           <t>36513</t>
         </is>
@@ -27634,7 +27664,7 @@
           <t>MEGLIC Jure</t>
         </is>
       </c>
-      <c r="U465" t="inlineStr">
+      <c r="X465" t="inlineStr">
         <is>
           <t>35590</t>
         </is>
@@ -27702,7 +27732,7 @@
           <t>PETERLIN Janos</t>
         </is>
       </c>
-      <c r="U466" t="inlineStr">
+      <c r="X466" t="inlineStr">
         <is>
           <t>36268</t>
         </is>
@@ -27770,7 +27800,7 @@
           <t>ALBREHT Martin</t>
         </is>
       </c>
-      <c r="U467" t="inlineStr">
+      <c r="X467" t="inlineStr">
         <is>
           <t>36898</t>
         </is>
@@ -27838,7 +27868,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U468" t="inlineStr">
+      <c r="X468" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -27906,7 +27936,7 @@
           <t>IVALDI Zeno</t>
         </is>
       </c>
-      <c r="U469" t="inlineStr">
+      <c r="X469" t="inlineStr">
         <is>
           <t>35480</t>
         </is>
@@ -27974,7 +28004,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U470" t="inlineStr">
+      <c r="X470" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -28042,7 +28072,7 @@
           <t>GLEJTEKOVA Simona</t>
         </is>
       </c>
-      <c r="U471" t="inlineStr">
+      <c r="X471" t="inlineStr">
         <is>
           <t>55166</t>
         </is>
@@ -28173,7 +28203,7 @@
           <t>GIBSON Eilidh</t>
         </is>
       </c>
-      <c r="U473" t="inlineStr">
+      <c r="X473" t="inlineStr">
         <is>
           <t>36708</t>
         </is>
@@ -28304,7 +28334,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U475" t="inlineStr">
+      <c r="X475" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -28372,7 +28402,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U476" t="inlineStr">
+      <c r="X476" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -28503,7 +28533,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U478" t="inlineStr">
+      <c r="X478" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -28571,7 +28601,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U479" t="inlineStr">
+      <c r="X479" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -28639,7 +28669,7 @@
           <t>JACQUET Claire</t>
         </is>
       </c>
-      <c r="U480" t="inlineStr">
+      <c r="X480" t="inlineStr">
         <is>
           <t>35684</t>
         </is>
@@ -28856,7 +28886,7 @@
           <t>CWIK Sara</t>
         </is>
       </c>
-      <c r="U484" t="inlineStr">
+      <c r="X484" t="inlineStr">
         <is>
           <t>43978</t>
         </is>
@@ -28967,7 +28997,7 @@
           <t>WEGMAN Martina</t>
         </is>
       </c>
-      <c r="U486" t="inlineStr">
+      <c r="X486" t="inlineStr">
         <is>
           <t>35345</t>
         </is>
@@ -29025,7 +29055,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U487" t="inlineStr">
+      <c r="X487" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -29083,7 +29113,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U488" t="inlineStr">
+      <c r="X488" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -29141,7 +29171,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U489" t="inlineStr">
+      <c r="X489" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -29199,7 +29229,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U490" t="inlineStr">
+      <c r="X490" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -29363,7 +29393,7 @@
           <t>KRAGELJ Ursa</t>
         </is>
       </c>
-      <c r="U493" t="inlineStr">
+      <c r="X493" t="inlineStr">
         <is>
           <t>36264</t>
         </is>
@@ -29421,7 +29451,7 @@
           <t>BOUZIDI Carole</t>
         </is>
       </c>
-      <c r="U494" t="inlineStr">
+      <c r="X494" t="inlineStr">
         <is>
           <t>35231</t>
         </is>
@@ -29479,7 +29509,7 @@
           <t>TROMPETER Caroline</t>
         </is>
       </c>
-      <c r="U495" t="inlineStr">
+      <c r="X495" t="inlineStr">
         <is>
           <t>39167</t>
         </is>
@@ -29537,7 +29567,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U496" t="inlineStr">
+      <c r="X496" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -29595,7 +29625,7 @@
           <t>MARTINEZ Marta</t>
         </is>
       </c>
-      <c r="U497" t="inlineStr">
+      <c r="X497" t="inlineStr">
         <is>
           <t>35760</t>
         </is>
@@ -29706,7 +29736,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U499" t="inlineStr">
+      <c r="X499" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -29764,7 +29794,7 @@
           <t>OBLINGER-PETERS Violetta</t>
         </is>
       </c>
-      <c r="U500" t="inlineStr">
+      <c r="X500" t="inlineStr">
         <is>
           <t>35289</t>
         </is>
@@ -29822,7 +29852,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U501" t="inlineStr">
+      <c r="X501" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -29880,7 +29910,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U502" t="inlineStr">
+      <c r="X502" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -29938,7 +29968,7 @@
           <t>MANGIN Estelle</t>
         </is>
       </c>
-      <c r="U503" t="inlineStr">
+      <c r="X503" t="inlineStr">
         <is>
           <t>35670</t>
         </is>
@@ -29996,7 +30026,7 @@
           <t>PENNIE Fiona</t>
         </is>
       </c>
-      <c r="U504" t="inlineStr">
+      <c r="X504" t="inlineStr">
         <is>
           <t>35638</t>
         </is>
@@ -30054,7 +30084,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U505" t="inlineStr">
+      <c r="X505" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -30112,7 +30142,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U506" t="inlineStr">
+      <c r="X506" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -30170,7 +30200,7 @@
           <t>GUIET Pauline</t>
         </is>
       </c>
-      <c r="U507" t="inlineStr">
+      <c r="X507" t="inlineStr">
         <is>
           <t>35493</t>
         </is>
@@ -30228,7 +30258,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U508" t="inlineStr">
+      <c r="X508" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -30286,7 +30316,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U509" t="inlineStr">
+      <c r="X509" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -30344,7 +30374,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U510" t="inlineStr">
+      <c r="X510" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -30402,7 +30432,7 @@
           <t>DUKATOVA Jana</t>
         </is>
       </c>
-      <c r="U511" t="inlineStr">
+      <c r="X511" t="inlineStr">
         <is>
           <t>35354</t>
         </is>
@@ -30460,7 +30490,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U512" t="inlineStr">
+      <c r="X512" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -30518,7 +30548,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U513" t="inlineStr">
+      <c r="X513" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -30581,12 +30611,12 @@
           <t>BETTGE Nico</t>
         </is>
       </c>
-      <c r="U514" t="inlineStr">
+      <c r="X514" t="inlineStr">
         <is>
           <t>35145</t>
         </is>
       </c>
-      <c r="V514" t="inlineStr">
+      <c r="Y514" t="inlineStr">
         <is>
           <t>35133</t>
         </is>
@@ -30649,12 +30679,12 @@
           <t>XIE Yuancong</t>
         </is>
       </c>
-      <c r="U515" t="inlineStr">
+      <c r="X515" t="inlineStr">
         <is>
           <t>42912</t>
         </is>
       </c>
-      <c r="V515" t="inlineStr">
+      <c r="Y515" t="inlineStr">
         <is>
           <t>72214</t>
         </is>
@@ -30717,12 +30747,12 @@
           <t>BATIK Jan</t>
         </is>
       </c>
-      <c r="U516" t="inlineStr">
+      <c r="X516" t="inlineStr">
         <is>
           <t>35368</t>
         </is>
       </c>
-      <c r="V516" t="inlineStr">
+      <c r="Y516" t="inlineStr">
         <is>
           <t>35367</t>
         </is>
@@ -30785,12 +30815,12 @@
           <t>DENG Xiao</t>
         </is>
       </c>
-      <c r="U517" t="inlineStr">
+      <c r="X517" t="inlineStr">
         <is>
           <t>42239</t>
         </is>
       </c>
-      <c r="V517" t="inlineStr">
+      <c r="Y517" t="inlineStr">
         <is>
           <t>42240</t>
         </is>
@@ -30853,12 +30883,12 @@
           <t>JANE Jakub</t>
         </is>
       </c>
-      <c r="U518" t="inlineStr">
+      <c r="X518" t="inlineStr">
         <is>
           <t>35060</t>
         </is>
       </c>
-      <c r="V518" t="inlineStr">
+      <c r="Y518" t="inlineStr">
         <is>
           <t>35061</t>
         </is>
@@ -30921,12 +30951,12 @@
           <t>CHEN Jin</t>
         </is>
       </c>
-      <c r="U519" t="inlineStr">
+      <c r="X519" t="inlineStr">
         <is>
           <t>42237</t>
         </is>
       </c>
-      <c r="V519" t="inlineStr">
+      <c r="Y519" t="inlineStr">
         <is>
           <t>42238</t>
         </is>
@@ -30989,12 +31019,12 @@
           <t>EICHFELD Casey</t>
         </is>
       </c>
-      <c r="U520" t="inlineStr">
+      <c r="X520" t="inlineStr">
         <is>
           <t>35068</t>
         </is>
       </c>
-      <c r="V520" t="inlineStr">
+      <c r="Y520" t="inlineStr">
         <is>
           <t>35067</t>
         </is>
@@ -31057,12 +31087,12 @@
           <t>OLIVEIRA Anderson</t>
         </is>
       </c>
-      <c r="U521" t="inlineStr">
+      <c r="X521" t="inlineStr">
         <is>
           <t>38018</t>
         </is>
       </c>
-      <c r="V521" t="inlineStr">
+      <c r="Y521" t="inlineStr">
         <is>
           <t>38020</t>
         </is>
@@ -31125,12 +31155,12 @@
           <t>MUELLER Kevin</t>
         </is>
       </c>
-      <c r="U522" t="inlineStr">
+      <c r="X522" t="inlineStr">
         <is>
           <t>35148</t>
         </is>
       </c>
-      <c r="V522" t="inlineStr">
+      <c r="Y522" t="inlineStr">
         <is>
           <t>35149</t>
         </is>
@@ -31193,12 +31223,12 @@
           <t>MAJERCZAK Grzegorz</t>
         </is>
       </c>
-      <c r="U523" t="inlineStr">
+      <c r="X523" t="inlineStr">
         <is>
           <t>35085</t>
         </is>
       </c>
-      <c r="V523" t="inlineStr">
+      <c r="Y523" t="inlineStr">
         <is>
           <t>35086</t>
         </is>
@@ -31261,12 +31291,12 @@
           <t>WERRO Simon</t>
         </is>
       </c>
-      <c r="U524" t="inlineStr">
+      <c r="X524" t="inlineStr">
         <is>
           <t>35347</t>
         </is>
       </c>
-      <c r="V524" t="inlineStr">
+      <c r="Y524" t="inlineStr">
         <is>
           <t>35424</t>
         </is>
@@ -31329,12 +31359,12 @@
           <t>CAILHOL Hugo</t>
         </is>
       </c>
-      <c r="U525" t="inlineStr">
+      <c r="X525" t="inlineStr">
         <is>
           <t>35476</t>
         </is>
       </c>
-      <c r="V525" t="inlineStr">
+      <c r="Y525" t="inlineStr">
         <is>
           <t>35491</t>
         </is>
@@ -31397,12 +31427,12 @@
           <t>BECKER Thomas</t>
         </is>
       </c>
-      <c r="U526" t="inlineStr">
+      <c r="X526" t="inlineStr">
         <is>
           <t>35139</t>
         </is>
       </c>
-      <c r="V526" t="inlineStr">
+      <c r="Y526" t="inlineStr">
         <is>
           <t>35143</t>
         </is>
@@ -31465,12 +31495,12 @@
           <t>SKANTAR Peter</t>
         </is>
       </c>
-      <c r="U527" t="inlineStr">
+      <c r="X527" t="inlineStr">
         <is>
           <t>35360</t>
         </is>
       </c>
-      <c r="V527" t="inlineStr">
+      <c r="Y527" t="inlineStr">
         <is>
           <t>35361</t>
         </is>
@@ -31533,12 +31563,12 @@
           <t>BRZEZINSKI Andrzej</t>
         </is>
       </c>
-      <c r="U528" t="inlineStr">
+      <c r="X528" t="inlineStr">
         <is>
           <t>35082</t>
         </is>
       </c>
-      <c r="V528" t="inlineStr">
+      <c r="Y528" t="inlineStr">
         <is>
           <t>35081</t>
         </is>
@@ -31601,12 +31631,12 @@
           <t>POCHWALA Marcin</t>
         </is>
       </c>
-      <c r="U529" t="inlineStr">
+      <c r="X529" t="inlineStr">
         <is>
           <t>35080</t>
         </is>
       </c>
-      <c r="V529" t="inlineStr">
+      <c r="Y529" t="inlineStr">
         <is>
           <t>35079</t>
         </is>
@@ -31669,12 +31699,12 @@
           <t>TALJAT Saso</t>
         </is>
       </c>
-      <c r="U530" t="inlineStr">
+      <c r="X530" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
       </c>
-      <c r="V530" t="inlineStr">
+      <c r="Y530" t="inlineStr">
         <is>
           <t>36270</t>
         </is>
@@ -31737,12 +31767,12 @@
           <t>VRZAN Jakub</t>
         </is>
       </c>
-      <c r="U531" t="inlineStr">
+      <c r="X531" t="inlineStr">
         <is>
           <t>35042</t>
         </is>
       </c>
-      <c r="V531" t="inlineStr">
+      <c r="Y531" t="inlineStr">
         <is>
           <t>35043</t>
         </is>
@@ -31805,12 +31835,12 @@
           <t>BISO Hugo</t>
         </is>
       </c>
-      <c r="U532" t="inlineStr">
+      <c r="X532" t="inlineStr">
         <is>
           <t>35403</t>
         </is>
       </c>
-      <c r="V532" t="inlineStr">
+      <c r="Y532" t="inlineStr">
         <is>
           <t>35229</t>
         </is>
@@ -31873,12 +31903,12 @@
           <t>LE RUYET Edern</t>
         </is>
       </c>
-      <c r="U533" t="inlineStr">
+      <c r="X533" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
       </c>
-      <c r="V533" t="inlineStr">
+      <c r="Y533" t="inlineStr">
         <is>
           <t>35379</t>
         </is>
@@ -31946,7 +31976,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U534" t="inlineStr">
+      <c r="X534" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -32077,7 +32107,7 @@
           <t>OBLINGER-PETERS Violetta</t>
         </is>
       </c>
-      <c r="U536" t="inlineStr">
+      <c r="X536" t="inlineStr">
         <is>
           <t>35289</t>
         </is>
@@ -32145,7 +32175,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U537" t="inlineStr">
+      <c r="X537" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -32213,7 +32243,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U538" t="inlineStr">
+      <c r="X538" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -32281,7 +32311,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U539" t="inlineStr">
+      <c r="X539" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -32349,7 +32379,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U540" t="inlineStr">
+      <c r="X540" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -32417,7 +32447,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U541" t="inlineStr">
+      <c r="X541" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -32485,7 +32515,7 @@
           <t>PENNIE Fiona</t>
         </is>
       </c>
-      <c r="U542" t="inlineStr">
+      <c r="X542" t="inlineStr">
         <is>
           <t>35638</t>
         </is>
@@ -32553,7 +32583,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U543" t="inlineStr">
+      <c r="X543" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -32626,12 +32656,12 @@
           <t>CAILHOL Hugo</t>
         </is>
       </c>
-      <c r="U544" t="inlineStr">
+      <c r="X544" t="inlineStr">
         <is>
           <t>35476</t>
         </is>
       </c>
-      <c r="V544" t="inlineStr">
+      <c r="Y544" t="inlineStr">
         <is>
           <t>35491</t>
         </is>
@@ -32704,12 +32734,12 @@
           <t>BRZEZINSKI Andrzej</t>
         </is>
       </c>
-      <c r="U545" t="inlineStr">
+      <c r="X545" t="inlineStr">
         <is>
           <t>35082</t>
         </is>
       </c>
-      <c r="V545" t="inlineStr">
+      <c r="Y545" t="inlineStr">
         <is>
           <t>35081</t>
         </is>
@@ -32782,12 +32812,12 @@
           <t>POCHWALA Marcin</t>
         </is>
       </c>
-      <c r="U546" t="inlineStr">
+      <c r="X546" t="inlineStr">
         <is>
           <t>35080</t>
         </is>
       </c>
-      <c r="V546" t="inlineStr">
+      <c r="Y546" t="inlineStr">
         <is>
           <t>35079</t>
         </is>
@@ -32860,12 +32890,12 @@
           <t>LE RUYET Edern</t>
         </is>
       </c>
-      <c r="U547" t="inlineStr">
+      <c r="X547" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
       </c>
-      <c r="V547" t="inlineStr">
+      <c r="Y547" t="inlineStr">
         <is>
           <t>35379</t>
         </is>
@@ -32938,12 +32968,12 @@
           <t>VRZAN Jakub</t>
         </is>
       </c>
-      <c r="U548" t="inlineStr">
+      <c r="X548" t="inlineStr">
         <is>
           <t>35042</t>
         </is>
       </c>
-      <c r="V548" t="inlineStr">
+      <c r="Y548" t="inlineStr">
         <is>
           <t>35043</t>
         </is>
@@ -33016,12 +33046,12 @@
           <t>WERRO Simon</t>
         </is>
       </c>
-      <c r="U549" t="inlineStr">
+      <c r="X549" t="inlineStr">
         <is>
           <t>35347</t>
         </is>
       </c>
-      <c r="V549" t="inlineStr">
+      <c r="Y549" t="inlineStr">
         <is>
           <t>35424</t>
         </is>
@@ -33094,12 +33124,12 @@
           <t>BATIK Jan</t>
         </is>
       </c>
-      <c r="U550" t="inlineStr">
+      <c r="X550" t="inlineStr">
         <is>
           <t>35368</t>
         </is>
       </c>
-      <c r="V550" t="inlineStr">
+      <c r="Y550" t="inlineStr">
         <is>
           <t>35367</t>
         </is>
@@ -33172,12 +33202,12 @@
           <t>JANE Jakub</t>
         </is>
       </c>
-      <c r="U551" t="inlineStr">
+      <c r="X551" t="inlineStr">
         <is>
           <t>35060</t>
         </is>
       </c>
-      <c r="V551" t="inlineStr">
+      <c r="Y551" t="inlineStr">
         <is>
           <t>35061</t>
         </is>
@@ -33250,12 +33280,12 @@
           <t>BISO Hugo</t>
         </is>
       </c>
-      <c r="U552" t="inlineStr">
+      <c r="X552" t="inlineStr">
         <is>
           <t>35403</t>
         </is>
       </c>
-      <c r="V552" t="inlineStr">
+      <c r="Y552" t="inlineStr">
         <is>
           <t>35229</t>
         </is>
@@ -33328,12 +33358,12 @@
           <t>SKANTAR Peter</t>
         </is>
       </c>
-      <c r="U553" t="inlineStr">
+      <c r="X553" t="inlineStr">
         <is>
           <t>35360</t>
         </is>
       </c>
-      <c r="V553" t="inlineStr">
+      <c r="Y553" t="inlineStr">
         <is>
           <t>35361</t>
         </is>

</xml_diff>